<commit_message>
fix(thoihieu): noi rong cot C va bo dinh dang vung F32:L34 duoi bang, chi giu all border
- Cot C 10.14 -> 13.43 (Excel 12.71): tieu de "Quet ma o / Buu cuc" TNR 12 dam het bi de chu.
- F32:L34 sheet Tong: Clear Formats (bo nen trang dac + can giua), roi All Borders net mong.
- Chi sua file mau; sheet data, cong thuc, merge, conditional format va zoom 70% giu nguyen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/AutoJMS/FullStack/UI/ThoiHieu/ThoiHieuKpi.template.xlsx
+++ b/src/AutoJMS/FullStack/UI/ThoiHieu/ThoiHieuKpi.template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" showInkAnnotation="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16CD85EC-980E-4911-A4D8-FB7A45254055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A98ACE5-16BE-4DAA-B39B-63AB23FCED2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="3645" windowWidth="21600" windowHeight="11835" xr2:uid="{47AA215E-EE30-4004-800A-4EDF6E1F8BAD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{47AA215E-EE30-4004-800A-4EDF6E1F8BAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Tổng" sheetId="1" r:id="rId1"/>
@@ -275,9 +275,9 @@
   <numFmts count="5">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0_ "/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="170" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0_ "/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -599,7 +599,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -626,7 +626,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -659,7 +658,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -673,12 +672,11 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="18" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -688,9 +686,6 @@
     <xf numFmtId="1" fontId="13" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -698,8 +693,23 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="18" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -724,21 +734,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1026,7 +1021,7 @@
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
     <col min="4" max="4" width="13.28515625" style="8" customWidth="1"/>
     <col min="5" max="5" width="31" customWidth="1"/>
     <col min="6" max="6" width="9.85546875" style="9" customWidth="1"/>
@@ -1034,166 +1029,166 @@
     <col min="8" max="8" width="11.42578125" style="9" customWidth="1"/>
     <col min="9" max="9" width="7.42578125" style="9" customWidth="1"/>
     <col min="10" max="10" width="10.85546875" customWidth="1"/>
-    <col min="11" max="11" width="8.140625" style="25" customWidth="1"/>
+    <col min="11" max="11" width="8.140625" style="24" customWidth="1"/>
     <col min="12" max="29" width="8.140625" style="9" customWidth="1"/>
     <col min="31" max="31" width="31" customWidth="1"/>
     <col min="33" max="33" width="28.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="81" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="L1" s="33">
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="L1" s="31">
         <v>3000</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="33">
+      <c r="N1" s="31">
         <v>2950</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="31">
+      <c r="P1" s="29">
         <v>2</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="Q1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="33">
+      <c r="R1" s="31">
         <v>15</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="S1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="34">
+      <c r="T1" s="32">
         <f>F31</f>
         <v>6888</v>
       </c>
-      <c r="U1" s="35" t="s">
+      <c r="U1" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="52">
+      <c r="V1" s="41">
         <f>T1*91%</f>
         <v>6268.08</v>
       </c>
-      <c r="W1" s="53"/>
-      <c r="X1" s="35" t="s">
+      <c r="W1" s="42"/>
+      <c r="X1" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="Y1" s="41">
+      <c r="Y1" s="43">
         <f>T1*90%</f>
         <v>6199.2</v>
       </c>
-      <c r="Z1" s="42"/>
-      <c r="AA1" s="43"/>
-      <c r="AB1" s="50" t="s">
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="45"/>
+      <c r="AB1" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="AC1" s="50" t="s">
+      <c r="AC1" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="AD1" s="49"/>
+      <c r="AD1" s="38"/>
     </row>
     <row r="2" spans="1:35" s="7" customFormat="1" ht="77.25" customHeight="1">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="M2" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="17" t="s">
+      <c r="N2" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="17" t="s">
+      <c r="O2" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="17" t="s">
+      <c r="P2" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="17" t="s">
+      <c r="Q2" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="17" t="s">
+      <c r="R2" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="17" t="s">
+      <c r="S2" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="T2" s="17" t="s">
+      <c r="T2" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="U2" s="17" t="s">
+      <c r="U2" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="V2" s="17" t="s">
+      <c r="V2" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="W2" s="17" t="s">
+      <c r="W2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="X2" s="17" t="s">
+      <c r="X2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="Y2" s="17" t="s">
+      <c r="Y2" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="Z2" s="17" t="s">
+      <c r="Z2" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="AA2" s="17" t="s">
+      <c r="AA2" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="AB2" s="50"/>
-      <c r="AC2" s="50"/>
-      <c r="AD2" s="49"/>
+      <c r="AB2" s="39"/>
+      <c r="AC2" s="39"/>
+      <c r="AD2" s="38"/>
       <c r="AE2"/>
       <c r="AF2"/>
       <c r="AG2"/>
@@ -1201,2740 +1196,2745 @@
       <c r="AI2"/>
     </row>
     <row r="3" spans="1:35" ht="15" customHeight="1">
-      <c r="A3" s="14">
+      <c r="A3" s="13">
         <v>1</v>
       </c>
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="21" t="s">
+      <c r="D3" s="13"/>
+      <c r="E3" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="13">
         <v>175</v>
       </c>
-      <c r="G3" s="23">
+      <c r="G3" s="22">
         <f t="shared" ref="G3:G30" si="0">F3*911/1000</f>
         <v>159.42500000000001</v>
       </c>
-      <c r="H3" s="23">
+      <c r="H3" s="22">
         <f>F3*90%</f>
         <v>157.5</v>
       </c>
-      <c r="I3" s="18">
+      <c r="I3" s="17">
         <f>SUM(K3:AA3)</f>
         <v>155</v>
       </c>
-      <c r="J3" s="32">
+      <c r="J3" s="30">
         <f>I3/F3</f>
         <v>0.88571428571428568</v>
       </c>
-      <c r="K3" s="19">
+      <c r="K3" s="18">
         <v>2</v>
       </c>
-      <c r="L3" s="19">
+      <c r="L3" s="18">
         <v>4</v>
       </c>
-      <c r="M3" s="19">
+      <c r="M3" s="18">
         <v>4</v>
       </c>
-      <c r="N3" s="19">
+      <c r="N3" s="18">
         <v>17</v>
       </c>
-      <c r="O3" s="19">
+      <c r="O3" s="18">
         <v>5</v>
       </c>
-      <c r="P3" s="19">
+      <c r="P3" s="18">
         <v>8</v>
       </c>
-      <c r="Q3" s="19">
+      <c r="Q3" s="18">
         <v>23</v>
       </c>
-      <c r="R3" s="19">
+      <c r="R3" s="18">
         <v>16</v>
       </c>
-      <c r="S3" s="19">
+      <c r="S3" s="18">
         <v>5</v>
       </c>
-      <c r="T3" s="19">
+      <c r="T3" s="18">
         <v>25</v>
       </c>
-      <c r="U3" s="19">
+      <c r="U3" s="18">
         <v>7</v>
       </c>
-      <c r="V3" s="19">
+      <c r="V3" s="18">
         <v>8</v>
       </c>
-      <c r="W3" s="19">
+      <c r="W3" s="18">
         <v>16</v>
       </c>
-      <c r="X3" s="19">
+      <c r="X3" s="18">
         <v>10</v>
       </c>
-      <c r="Y3" s="19">
+      <c r="Y3" s="18">
         <v>3</v>
       </c>
-      <c r="Z3" s="19">
+      <c r="Z3" s="18">
         <v>2</v>
       </c>
-      <c r="AA3" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="40">
+      <c r="AA3" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="37">
         <f>G3-I3</f>
         <v>4.4250000000000114</v>
       </c>
-      <c r="AC3" s="40">
+      <c r="AC3" s="37">
         <f>H3-I3</f>
         <v>2.5</v>
       </c>
-      <c r="AD3" s="37"/>
+      <c r="AD3" s="34"/>
     </row>
     <row r="4" spans="1:35" ht="15" customHeight="1">
-      <c r="A4" s="14">
+      <c r="A4" s="13">
         <v>2</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="14" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="21" t="s">
+      <c r="D4" s="13"/>
+      <c r="E4" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="14">
+      <c r="F4" s="13">
         <v>217</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="22">
         <f t="shared" si="0"/>
         <v>197.68700000000001</v>
       </c>
-      <c r="H4" s="23">
+      <c r="H4" s="22">
         <f t="shared" ref="H4:H27" si="1">F4*90%</f>
         <v>195.3</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="17">
         <f t="shared" ref="I4:I27" si="2">SUM(K4:AA4)</f>
         <v>215</v>
       </c>
-      <c r="J4" s="32">
+      <c r="J4" s="30">
         <f t="shared" ref="J4:J27" si="3">I4/F4</f>
         <v>0.99078341013824889</v>
       </c>
-      <c r="K4" s="19">
-        <v>0</v>
-      </c>
-      <c r="L4" s="19">
+      <c r="K4" s="18">
+        <v>0</v>
+      </c>
+      <c r="L4" s="18">
         <v>26</v>
       </c>
-      <c r="M4" s="19">
+      <c r="M4" s="18">
         <v>19</v>
       </c>
-      <c r="N4" s="19">
+      <c r="N4" s="18">
         <v>13</v>
       </c>
-      <c r="O4" s="19">
+      <c r="O4" s="18">
         <v>5</v>
       </c>
-      <c r="P4" s="19">
+      <c r="P4" s="18">
         <v>2</v>
       </c>
-      <c r="Q4" s="19">
+      <c r="Q4" s="18">
         <v>23</v>
       </c>
-      <c r="R4" s="19">
+      <c r="R4" s="18">
         <v>26</v>
       </c>
-      <c r="S4" s="19">
+      <c r="S4" s="18">
         <v>17</v>
       </c>
-      <c r="T4" s="19">
+      <c r="T4" s="18">
         <v>1</v>
       </c>
-      <c r="U4" s="19">
+      <c r="U4" s="18">
         <v>23</v>
       </c>
-      <c r="V4" s="19">
+      <c r="V4" s="18">
         <v>4</v>
       </c>
-      <c r="W4" s="19">
+      <c r="W4" s="18">
         <v>29</v>
       </c>
-      <c r="X4" s="19">
+      <c r="X4" s="18">
         <v>22</v>
       </c>
-      <c r="Y4" s="19">
+      <c r="Y4" s="18">
         <v>4</v>
       </c>
-      <c r="Z4" s="19">
+      <c r="Z4" s="18">
         <v>1</v>
       </c>
-      <c r="AA4" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="40">
+      <c r="AA4" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="37">
         <f t="shared" ref="AB4:AB30" si="4">G4-I4</f>
         <v>-17.312999999999988</v>
       </c>
-      <c r="AC4" s="40">
+      <c r="AC4" s="37">
         <f t="shared" ref="AC4:AC30" si="5">H4-I4</f>
         <v>-19.699999999999989</v>
       </c>
-      <c r="AD4" s="37"/>
+      <c r="AD4" s="34"/>
     </row>
     <row r="5" spans="1:35" ht="14.45" customHeight="1">
-      <c r="A5" s="14">
+      <c r="A5" s="13">
         <v>3</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="14" t="s">
+      <c r="B5" s="40"/>
+      <c r="C5" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="21" t="s">
+      <c r="D5" s="13"/>
+      <c r="E5" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="14">
+      <c r="F5" s="13">
         <v>198</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="22">
         <f t="shared" si="0"/>
         <v>180.37799999999999</v>
       </c>
-      <c r="H5" s="23">
+      <c r="H5" s="22">
         <f t="shared" si="1"/>
         <v>178.20000000000002</v>
       </c>
-      <c r="I5" s="18">
+      <c r="I5" s="17">
         <f t="shared" si="2"/>
         <v>185</v>
       </c>
-      <c r="J5" s="32">
+      <c r="J5" s="30">
         <f t="shared" si="3"/>
         <v>0.93434343434343436</v>
       </c>
-      <c r="K5" s="19">
-        <v>0</v>
-      </c>
-      <c r="L5" s="19">
+      <c r="K5" s="18">
+        <v>0</v>
+      </c>
+      <c r="L5" s="18">
         <v>19</v>
       </c>
-      <c r="M5" s="19">
+      <c r="M5" s="18">
         <v>27</v>
       </c>
-      <c r="N5" s="19">
-        <v>0</v>
-      </c>
-      <c r="O5" s="19">
+      <c r="N5" s="18">
+        <v>0</v>
+      </c>
+      <c r="O5" s="18">
         <v>17</v>
       </c>
-      <c r="P5" s="19">
+      <c r="P5" s="18">
         <v>26</v>
       </c>
-      <c r="Q5" s="19">
+      <c r="Q5" s="18">
         <v>24</v>
       </c>
-      <c r="R5" s="19">
+      <c r="R5" s="18">
         <v>12</v>
       </c>
-      <c r="S5" s="19">
+      <c r="S5" s="18">
         <v>4</v>
       </c>
-      <c r="T5" s="19">
-        <v>0</v>
-      </c>
-      <c r="U5" s="19">
+      <c r="T5" s="18">
+        <v>0</v>
+      </c>
+      <c r="U5" s="18">
         <v>1</v>
       </c>
-      <c r="V5" s="19">
+      <c r="V5" s="18">
         <v>25</v>
       </c>
-      <c r="W5" s="19">
+      <c r="W5" s="18">
         <v>20</v>
       </c>
-      <c r="X5" s="19">
+      <c r="X5" s="18">
         <v>3</v>
       </c>
-      <c r="Y5" s="19">
+      <c r="Y5" s="18">
         <v>1</v>
       </c>
-      <c r="Z5" s="19">
+      <c r="Z5" s="18">
         <v>6</v>
       </c>
-      <c r="AA5" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="40">
+      <c r="AA5" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="37">
         <f t="shared" si="4"/>
         <v>-4.6220000000000141</v>
       </c>
-      <c r="AC5" s="40">
+      <c r="AC5" s="37">
         <f t="shared" si="5"/>
         <v>-6.7999999999999829</v>
       </c>
-      <c r="AD5" s="37"/>
+      <c r="AD5" s="34"/>
     </row>
     <row r="6" spans="1:35" ht="14.45" customHeight="1">
-      <c r="A6" s="14">
+      <c r="A6" s="13">
         <v>4</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="14" t="s">
+      <c r="B6" s="40"/>
+      <c r="C6" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="21" t="s">
+      <c r="D6" s="13"/>
+      <c r="E6" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="13">
         <v>148</v>
       </c>
-      <c r="G6" s="23">
+      <c r="G6" s="22">
         <f t="shared" si="0"/>
         <v>134.828</v>
       </c>
-      <c r="H6" s="23">
+      <c r="H6" s="22">
         <f t="shared" si="1"/>
         <v>133.20000000000002</v>
       </c>
-      <c r="I6" s="18">
+      <c r="I6" s="17">
         <f t="shared" si="2"/>
         <v>133</v>
       </c>
-      <c r="J6" s="32">
+      <c r="J6" s="30">
         <f t="shared" si="3"/>
         <v>0.89864864864864868</v>
       </c>
-      <c r="K6" s="19">
+      <c r="K6" s="18">
         <v>1</v>
       </c>
-      <c r="L6" s="19">
+      <c r="L6" s="18">
         <v>4</v>
       </c>
-      <c r="M6" s="19">
+      <c r="M6" s="18">
         <v>1</v>
       </c>
-      <c r="N6" s="19">
+      <c r="N6" s="18">
         <v>19</v>
       </c>
-      <c r="O6" s="19">
+      <c r="O6" s="18">
         <v>17</v>
       </c>
-      <c r="P6" s="19">
+      <c r="P6" s="18">
         <v>1</v>
       </c>
-      <c r="Q6" s="19">
+      <c r="Q6" s="18">
         <v>13</v>
       </c>
-      <c r="R6" s="19">
+      <c r="R6" s="18">
         <v>23</v>
       </c>
-      <c r="S6" s="19">
+      <c r="S6" s="18">
         <v>20</v>
       </c>
-      <c r="T6" s="19">
+      <c r="T6" s="18">
         <v>7</v>
       </c>
-      <c r="U6" s="19">
-        <v>0</v>
-      </c>
-      <c r="V6" s="19">
+      <c r="U6" s="18">
+        <v>0</v>
+      </c>
+      <c r="V6" s="18">
         <v>12</v>
       </c>
-      <c r="W6" s="19">
+      <c r="W6" s="18">
         <v>8</v>
       </c>
-      <c r="X6" s="19">
+      <c r="X6" s="18">
         <v>2</v>
       </c>
-      <c r="Y6" s="19">
+      <c r="Y6" s="18">
         <v>5</v>
       </c>
-      <c r="Z6" s="19">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="40">
+      <c r="Z6" s="18">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="37">
         <f t="shared" si="4"/>
         <v>1.828000000000003</v>
       </c>
-      <c r="AC6" s="40">
+      <c r="AC6" s="37">
         <f t="shared" si="5"/>
         <v>0.20000000000001705</v>
       </c>
-      <c r="AD6" s="37"/>
+      <c r="AD6" s="34"/>
     </row>
     <row r="7" spans="1:35" ht="14.45" customHeight="1">
-      <c r="A7" s="14">
+      <c r="A7" s="13">
         <v>5</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="14" t="s">
+      <c r="B7" s="40"/>
+      <c r="C7" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="21" t="s">
+      <c r="D7" s="13"/>
+      <c r="E7" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="13">
         <v>218</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="22">
         <f t="shared" si="0"/>
         <v>198.59800000000001</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="22">
         <f t="shared" si="1"/>
         <v>196.20000000000002</v>
       </c>
-      <c r="I7" s="18">
+      <c r="I7" s="17">
         <f t="shared" si="2"/>
         <v>189</v>
       </c>
-      <c r="J7" s="32">
+      <c r="J7" s="30">
         <f t="shared" si="3"/>
         <v>0.8669724770642202</v>
       </c>
-      <c r="K7" s="19">
-        <v>0</v>
-      </c>
-      <c r="L7" s="19">
+      <c r="K7" s="18">
+        <v>0</v>
+      </c>
+      <c r="L7" s="18">
         <v>26</v>
       </c>
-      <c r="M7" s="19">
+      <c r="M7" s="18">
         <v>14</v>
       </c>
-      <c r="N7" s="19">
+      <c r="N7" s="18">
         <v>16</v>
       </c>
-      <c r="O7" s="19">
+      <c r="O7" s="18">
         <v>16</v>
       </c>
-      <c r="P7" s="19">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="19">
+      <c r="P7" s="18">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="18">
         <v>27</v>
       </c>
-      <c r="R7" s="19">
-        <v>0</v>
-      </c>
-      <c r="S7" s="19">
-        <v>0</v>
-      </c>
-      <c r="T7" s="19">
+      <c r="R7" s="18">
+        <v>0</v>
+      </c>
+      <c r="S7" s="18">
+        <v>0</v>
+      </c>
+      <c r="T7" s="18">
         <v>2</v>
       </c>
-      <c r="U7" s="19">
+      <c r="U7" s="18">
         <v>21</v>
       </c>
-      <c r="V7" s="19">
+      <c r="V7" s="18">
         <v>1</v>
       </c>
-      <c r="W7" s="19">
+      <c r="W7" s="18">
         <v>30</v>
       </c>
-      <c r="X7" s="19">
+      <c r="X7" s="18">
         <v>30</v>
       </c>
-      <c r="Y7" s="19">
+      <c r="Y7" s="18">
         <v>3</v>
       </c>
-      <c r="Z7" s="19">
+      <c r="Z7" s="18">
         <v>3</v>
       </c>
-      <c r="AA7" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="40">
+      <c r="AA7" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="37">
         <f t="shared" si="4"/>
         <v>9.5980000000000132</v>
       </c>
-      <c r="AC7" s="40">
+      <c r="AC7" s="37">
         <f t="shared" si="5"/>
         <v>7.2000000000000171</v>
       </c>
-      <c r="AD7" s="37"/>
+      <c r="AD7" s="34"/>
     </row>
     <row r="8" spans="1:35" ht="14.45" customHeight="1">
-      <c r="A8" s="14">
+      <c r="A8" s="13">
         <v>6</v>
       </c>
-      <c r="B8" s="51"/>
-      <c r="C8" s="14" t="s">
+      <c r="B8" s="40"/>
+      <c r="C8" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="21" t="s">
+      <c r="D8" s="13"/>
+      <c r="E8" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="13">
         <v>243</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="22">
         <f t="shared" si="0"/>
         <v>221.37299999999999</v>
       </c>
-      <c r="H8" s="23">
+      <c r="H8" s="22">
         <f t="shared" si="1"/>
         <v>218.70000000000002</v>
       </c>
-      <c r="I8" s="18">
+      <c r="I8" s="17">
         <f t="shared" si="2"/>
         <v>234</v>
       </c>
-      <c r="J8" s="32">
+      <c r="J8" s="30">
         <f t="shared" si="3"/>
         <v>0.96296296296296291</v>
       </c>
-      <c r="K8" s="19">
-        <v>0</v>
-      </c>
-      <c r="L8" s="19">
+      <c r="K8" s="18">
+        <v>0</v>
+      </c>
+      <c r="L8" s="18">
         <v>12</v>
       </c>
-      <c r="M8" s="19">
+      <c r="M8" s="18">
         <v>4</v>
       </c>
-      <c r="N8" s="19">
+      <c r="N8" s="18">
         <v>14</v>
       </c>
-      <c r="O8" s="19">
+      <c r="O8" s="18">
         <v>26</v>
       </c>
-      <c r="P8" s="19">
+      <c r="P8" s="18">
         <v>17</v>
       </c>
-      <c r="Q8" s="19">
+      <c r="Q8" s="18">
         <v>13</v>
       </c>
-      <c r="R8" s="19">
+      <c r="R8" s="18">
         <v>9</v>
       </c>
-      <c r="S8" s="19">
+      <c r="S8" s="18">
         <v>29</v>
       </c>
-      <c r="T8" s="19">
+      <c r="T8" s="18">
         <v>19</v>
       </c>
-      <c r="U8" s="19">
+      <c r="U8" s="18">
         <v>24</v>
       </c>
-      <c r="V8" s="19">
-        <v>0</v>
-      </c>
-      <c r="W8" s="19">
+      <c r="V8" s="18">
+        <v>0</v>
+      </c>
+      <c r="W8" s="18">
         <v>29</v>
       </c>
-      <c r="X8" s="19">
+      <c r="X8" s="18">
         <v>31</v>
       </c>
-      <c r="Y8" s="19">
+      <c r="Y8" s="18">
         <v>2</v>
       </c>
-      <c r="Z8" s="19">
+      <c r="Z8" s="18">
         <v>5</v>
       </c>
-      <c r="AA8" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="40">
+      <c r="AA8" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="37">
         <f t="shared" si="4"/>
         <v>-12.62700000000001</v>
       </c>
-      <c r="AC8" s="40">
+      <c r="AC8" s="37">
         <f t="shared" si="5"/>
         <v>-15.299999999999983</v>
       </c>
-      <c r="AD8" s="37"/>
+      <c r="AD8" s="34"/>
     </row>
     <row r="9" spans="1:35" ht="15" customHeight="1">
-      <c r="A9" s="14">
+      <c r="A9" s="13">
         <v>7</v>
       </c>
-      <c r="B9" s="51"/>
-      <c r="C9" s="14" t="s">
+      <c r="B9" s="40"/>
+      <c r="C9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="21" t="s">
+      <c r="D9" s="13"/>
+      <c r="E9" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="13">
         <v>257</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="22">
         <f t="shared" si="0"/>
         <v>234.12700000000001</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="22">
         <f t="shared" si="1"/>
         <v>231.3</v>
       </c>
-      <c r="I9" s="18">
+      <c r="I9" s="17">
         <f t="shared" si="2"/>
         <v>221</v>
       </c>
-      <c r="J9" s="32">
+      <c r="J9" s="30">
         <f t="shared" si="3"/>
         <v>0.8599221789883269</v>
       </c>
-      <c r="K9" s="19">
-        <v>0</v>
-      </c>
-      <c r="L9" s="19">
+      <c r="K9" s="18">
+        <v>0</v>
+      </c>
+      <c r="L9" s="18">
         <v>14</v>
       </c>
-      <c r="M9" s="19">
+      <c r="M9" s="18">
         <v>10</v>
       </c>
-      <c r="N9" s="19">
+      <c r="N9" s="18">
         <v>25</v>
       </c>
-      <c r="O9" s="19">
+      <c r="O9" s="18">
         <v>4</v>
       </c>
-      <c r="P9" s="19">
+      <c r="P9" s="18">
         <v>4</v>
       </c>
-      <c r="Q9" s="19">
+      <c r="Q9" s="18">
         <v>7</v>
       </c>
-      <c r="R9" s="19">
+      <c r="R9" s="18">
         <v>19</v>
       </c>
-      <c r="S9" s="19">
+      <c r="S9" s="18">
         <v>16</v>
       </c>
-      <c r="T9" s="19">
+      <c r="T9" s="18">
         <v>32</v>
       </c>
-      <c r="U9" s="19">
+      <c r="U9" s="18">
         <v>25</v>
       </c>
-      <c r="V9" s="19">
+      <c r="V9" s="18">
         <v>22</v>
       </c>
-      <c r="W9" s="19">
+      <c r="W9" s="18">
         <v>23</v>
       </c>
-      <c r="X9" s="19">
+      <c r="X9" s="18">
         <v>9</v>
       </c>
-      <c r="Y9" s="19">
+      <c r="Y9" s="18">
         <v>4</v>
       </c>
-      <c r="Z9" s="19">
+      <c r="Z9" s="18">
         <v>7</v>
       </c>
-      <c r="AA9" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB9" s="40">
+      <c r="AA9" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="37">
         <f t="shared" si="4"/>
         <v>13.12700000000001</v>
       </c>
-      <c r="AC9" s="40">
+      <c r="AC9" s="37">
         <f t="shared" si="5"/>
         <v>10.300000000000011</v>
       </c>
-      <c r="AD9" s="37"/>
+      <c r="AD9" s="34"/>
     </row>
     <row r="10" spans="1:35" ht="15" customHeight="1">
-      <c r="A10" s="14">
+      <c r="A10" s="13">
         <v>8</v>
       </c>
-      <c r="B10" s="51"/>
-      <c r="C10" s="14" t="s">
+      <c r="B10" s="40"/>
+      <c r="C10" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="21" t="s">
+      <c r="D10" s="13"/>
+      <c r="E10" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="13">
         <v>169</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="22">
         <f t="shared" si="0"/>
         <v>153.959</v>
       </c>
-      <c r="H10" s="23">
+      <c r="H10" s="22">
         <f t="shared" si="1"/>
         <v>152.1</v>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="17">
         <f t="shared" si="2"/>
         <v>142</v>
       </c>
-      <c r="J10" s="32">
+      <c r="J10" s="30">
         <f t="shared" si="3"/>
         <v>0.84023668639053251</v>
       </c>
-      <c r="K10" s="19">
-        <v>0</v>
-      </c>
-      <c r="L10" s="19">
+      <c r="K10" s="18">
+        <v>0</v>
+      </c>
+      <c r="L10" s="18">
         <v>11</v>
       </c>
-      <c r="M10" s="19">
+      <c r="M10" s="18">
         <v>30</v>
       </c>
-      <c r="N10" s="19">
-        <v>0</v>
-      </c>
-      <c r="O10" s="19">
+      <c r="N10" s="18">
+        <v>0</v>
+      </c>
+      <c r="O10" s="18">
         <v>7</v>
       </c>
-      <c r="P10" s="19">
+      <c r="P10" s="18">
         <v>8</v>
       </c>
-      <c r="Q10" s="19">
+      <c r="Q10" s="18">
         <v>1</v>
       </c>
-      <c r="R10" s="19">
+      <c r="R10" s="18">
         <v>7</v>
       </c>
-      <c r="S10" s="19">
+      <c r="S10" s="18">
         <v>19</v>
       </c>
-      <c r="T10" s="19">
+      <c r="T10" s="18">
         <v>13</v>
       </c>
-      <c r="U10" s="19">
+      <c r="U10" s="18">
         <v>3</v>
       </c>
-      <c r="V10" s="19">
+      <c r="V10" s="18">
         <v>32</v>
       </c>
-      <c r="W10" s="19">
+      <c r="W10" s="18">
         <v>4</v>
       </c>
-      <c r="X10" s="19">
+      <c r="X10" s="18">
         <v>3</v>
       </c>
-      <c r="Y10" s="19">
+      <c r="Y10" s="18">
         <v>2</v>
       </c>
-      <c r="Z10" s="19">
+      <c r="Z10" s="18">
         <v>2</v>
       </c>
-      <c r="AA10" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="40">
+      <c r="AA10" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="37">
         <f t="shared" si="4"/>
         <v>11.959000000000003</v>
       </c>
-      <c r="AC10" s="40">
+      <c r="AC10" s="37">
         <f t="shared" si="5"/>
         <v>10.099999999999994</v>
       </c>
-      <c r="AD10" s="37"/>
+      <c r="AD10" s="34"/>
     </row>
     <row r="11" spans="1:35" ht="15" customHeight="1">
-      <c r="A11" s="14">
+      <c r="A11" s="13">
         <v>9</v>
       </c>
-      <c r="B11" s="51"/>
-      <c r="C11" s="14" t="s">
+      <c r="B11" s="40"/>
+      <c r="C11" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="21" t="s">
+      <c r="D11" s="13"/>
+      <c r="E11" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="14">
+      <c r="F11" s="13">
         <v>217</v>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="22">
         <f t="shared" si="0"/>
         <v>197.68700000000001</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="22">
         <f t="shared" si="1"/>
         <v>195.3</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="17">
         <f t="shared" si="2"/>
         <v>205</v>
       </c>
-      <c r="J11" s="32">
+      <c r="J11" s="30">
         <f t="shared" si="3"/>
         <v>0.9447004608294931</v>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="18">
         <v>2</v>
       </c>
-      <c r="L11" s="19">
-        <v>0</v>
-      </c>
-      <c r="M11" s="19">
+      <c r="L11" s="18">
+        <v>0</v>
+      </c>
+      <c r="M11" s="18">
         <v>1</v>
       </c>
-      <c r="N11" s="19">
+      <c r="N11" s="18">
         <v>27</v>
       </c>
-      <c r="O11" s="19">
+      <c r="O11" s="18">
         <v>29</v>
       </c>
-      <c r="P11" s="19">
+      <c r="P11" s="18">
         <v>7</v>
       </c>
-      <c r="Q11" s="19">
+      <c r="Q11" s="18">
         <v>30</v>
       </c>
-      <c r="R11" s="19">
+      <c r="R11" s="18">
         <v>27</v>
       </c>
-      <c r="S11" s="19">
+      <c r="S11" s="18">
         <v>9</v>
       </c>
-      <c r="T11" s="19">
+      <c r="T11" s="18">
         <v>17</v>
       </c>
-      <c r="U11" s="19">
+      <c r="U11" s="18">
         <v>20</v>
       </c>
-      <c r="V11" s="19">
+      <c r="V11" s="18">
         <v>20</v>
       </c>
-      <c r="W11" s="19">
+      <c r="W11" s="18">
         <v>6</v>
       </c>
-      <c r="X11" s="19">
+      <c r="X11" s="18">
         <v>9</v>
       </c>
-      <c r="Y11" s="19">
+      <c r="Y11" s="18">
         <v>1</v>
       </c>
-      <c r="Z11" s="19">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="40">
+      <c r="Z11" s="18">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="37">
         <f t="shared" si="4"/>
         <v>-7.3129999999999882</v>
       </c>
-      <c r="AC11" s="40">
+      <c r="AC11" s="37">
         <f t="shared" si="5"/>
         <v>-9.6999999999999886</v>
       </c>
-      <c r="AD11" s="37"/>
+      <c r="AD11" s="34"/>
     </row>
     <row r="12" spans="1:35" ht="15" customHeight="1">
-      <c r="A12" s="14">
+      <c r="A12" s="13">
         <v>10</v>
       </c>
-      <c r="B12" s="51"/>
-      <c r="C12" s="14" t="s">
+      <c r="B12" s="40"/>
+      <c r="C12" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="14"/>
-      <c r="E12" s="21" t="s">
+      <c r="D12" s="13"/>
+      <c r="E12" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="F12" s="14">
+      <c r="F12" s="13">
         <v>292</v>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="22">
         <f t="shared" si="0"/>
         <v>266.012</v>
       </c>
-      <c r="H12" s="23">
+      <c r="H12" s="22">
         <f t="shared" si="1"/>
         <v>262.8</v>
       </c>
-      <c r="I12" s="18">
+      <c r="I12" s="17">
         <f t="shared" si="2"/>
         <v>235</v>
       </c>
-      <c r="J12" s="32">
+      <c r="J12" s="30">
         <f t="shared" si="3"/>
         <v>0.8047945205479452</v>
       </c>
-      <c r="K12" s="19">
+      <c r="K12" s="18">
         <v>2</v>
       </c>
-      <c r="L12" s="19">
+      <c r="L12" s="18">
         <v>32</v>
       </c>
-      <c r="M12" s="19">
+      <c r="M12" s="18">
         <v>25</v>
       </c>
-      <c r="N12" s="19">
+      <c r="N12" s="18">
         <v>4</v>
       </c>
-      <c r="O12" s="19">
+      <c r="O12" s="18">
         <v>29</v>
       </c>
-      <c r="P12" s="19">
+      <c r="P12" s="18">
         <v>6</v>
       </c>
-      <c r="Q12" s="19">
+      <c r="Q12" s="18">
         <v>9</v>
       </c>
-      <c r="R12" s="19">
+      <c r="R12" s="18">
         <v>18</v>
       </c>
-      <c r="S12" s="19">
+      <c r="S12" s="18">
         <v>18</v>
       </c>
-      <c r="T12" s="19">
+      <c r="T12" s="18">
         <v>23</v>
       </c>
-      <c r="U12" s="19">
+      <c r="U12" s="18">
         <v>4</v>
       </c>
-      <c r="V12" s="19">
+      <c r="V12" s="18">
         <v>19</v>
       </c>
-      <c r="W12" s="19">
+      <c r="W12" s="18">
         <v>12</v>
       </c>
-      <c r="X12" s="19">
+      <c r="X12" s="18">
         <v>29</v>
       </c>
-      <c r="Y12" s="19">
+      <c r="Y12" s="18">
         <v>3</v>
       </c>
-      <c r="Z12" s="19">
+      <c r="Z12" s="18">
         <v>2</v>
       </c>
-      <c r="AA12" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="40">
+      <c r="AA12" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="37">
         <f t="shared" si="4"/>
         <v>31.012</v>
       </c>
-      <c r="AC12" s="40">
+      <c r="AC12" s="37">
         <f t="shared" si="5"/>
         <v>27.800000000000011</v>
       </c>
-      <c r="AD12" s="37"/>
+      <c r="AD12" s="34"/>
     </row>
     <row r="13" spans="1:35" ht="15" customHeight="1">
-      <c r="A13" s="14">
+      <c r="A13" s="13">
         <v>11</v>
       </c>
-      <c r="B13" s="51"/>
-      <c r="C13" s="14" t="s">
+      <c r="B13" s="40"/>
+      <c r="C13" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="21" t="s">
+      <c r="D13" s="13"/>
+      <c r="E13" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="F13" s="14">
+      <c r="F13" s="13">
         <v>251</v>
       </c>
-      <c r="G13" s="23">
+      <c r="G13" s="22">
         <f t="shared" si="0"/>
         <v>228.661</v>
       </c>
-      <c r="H13" s="23">
+      <c r="H13" s="22">
         <f t="shared" si="1"/>
         <v>225.9</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="17">
         <f t="shared" si="2"/>
         <v>205</v>
       </c>
-      <c r="J13" s="32">
+      <c r="J13" s="30">
         <f t="shared" si="3"/>
         <v>0.81673306772908372</v>
       </c>
-      <c r="K13" s="19">
+      <c r="K13" s="18">
         <v>1</v>
       </c>
-      <c r="L13" s="19">
+      <c r="L13" s="18">
         <v>17</v>
       </c>
-      <c r="M13" s="19">
+      <c r="M13" s="18">
         <v>31</v>
       </c>
-      <c r="N13" s="19">
+      <c r="N13" s="18">
         <v>26</v>
       </c>
-      <c r="O13" s="19">
+      <c r="O13" s="18">
         <v>4</v>
       </c>
-      <c r="P13" s="19">
+      <c r="P13" s="18">
         <v>3</v>
       </c>
-      <c r="Q13" s="19">
-        <v>0</v>
-      </c>
-      <c r="R13" s="19">
+      <c r="Q13" s="18">
+        <v>0</v>
+      </c>
+      <c r="R13" s="18">
         <v>6</v>
       </c>
-      <c r="S13" s="19">
+      <c r="S13" s="18">
         <v>31</v>
       </c>
-      <c r="T13" s="19">
+      <c r="T13" s="18">
         <v>23</v>
       </c>
-      <c r="U13" s="19">
+      <c r="U13" s="18">
         <v>13</v>
       </c>
-      <c r="V13" s="19">
+      <c r="V13" s="18">
         <v>19</v>
       </c>
-      <c r="W13" s="19">
+      <c r="W13" s="18">
         <v>13</v>
       </c>
-      <c r="X13" s="19">
+      <c r="X13" s="18">
         <v>4</v>
       </c>
-      <c r="Y13" s="19">
+      <c r="Y13" s="18">
         <v>7</v>
       </c>
-      <c r="Z13" s="19">
+      <c r="Z13" s="18">
         <v>7</v>
       </c>
-      <c r="AA13" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="40">
+      <c r="AA13" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="37">
         <f t="shared" si="4"/>
         <v>23.661000000000001</v>
       </c>
-      <c r="AC13" s="40">
+      <c r="AC13" s="37">
         <f t="shared" si="5"/>
         <v>20.900000000000006</v>
       </c>
-      <c r="AD13" s="37"/>
+      <c r="AD13" s="34"/>
     </row>
     <row r="14" spans="1:35" ht="15" customHeight="1">
-      <c r="A14" s="14">
+      <c r="A14" s="13">
         <v>12</v>
       </c>
-      <c r="B14" s="51"/>
-      <c r="C14" s="14" t="s">
+      <c r="B14" s="40"/>
+      <c r="C14" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="21" t="s">
+      <c r="D14" s="13"/>
+      <c r="E14" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="13">
         <v>268</v>
       </c>
-      <c r="G14" s="23">
+      <c r="G14" s="22">
         <f t="shared" si="0"/>
         <v>244.148</v>
       </c>
-      <c r="H14" s="23">
+      <c r="H14" s="22">
         <f t="shared" si="1"/>
         <v>241.20000000000002</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="17">
         <f t="shared" si="2"/>
         <v>254</v>
       </c>
-      <c r="J14" s="32">
+      <c r="J14" s="30">
         <f t="shared" si="3"/>
         <v>0.94776119402985071</v>
       </c>
-      <c r="K14" s="19">
-        <v>0</v>
-      </c>
-      <c r="L14" s="19">
+      <c r="K14" s="18">
+        <v>0</v>
+      </c>
+      <c r="L14" s="18">
         <v>11</v>
       </c>
-      <c r="M14" s="19">
+      <c r="M14" s="18">
         <v>17</v>
       </c>
-      <c r="N14" s="19">
+      <c r="N14" s="18">
         <v>20</v>
       </c>
-      <c r="O14" s="19">
+      <c r="O14" s="18">
         <v>31</v>
       </c>
-      <c r="P14" s="19">
+      <c r="P14" s="18">
         <v>27</v>
       </c>
-      <c r="Q14" s="19">
+      <c r="Q14" s="18">
         <v>24</v>
       </c>
-      <c r="R14" s="19">
+      <c r="R14" s="18">
         <v>9</v>
       </c>
-      <c r="S14" s="19">
+      <c r="S14" s="18">
         <v>11</v>
       </c>
-      <c r="T14" s="19">
+      <c r="T14" s="18">
         <v>17</v>
       </c>
-      <c r="U14" s="19">
+      <c r="U14" s="18">
         <v>26</v>
       </c>
-      <c r="V14" s="19">
+      <c r="V14" s="18">
         <v>8</v>
       </c>
-      <c r="W14" s="19">
+      <c r="W14" s="18">
         <v>29</v>
       </c>
-      <c r="X14" s="19">
+      <c r="X14" s="18">
         <v>21</v>
       </c>
-      <c r="Y14" s="19">
+      <c r="Y14" s="18">
         <v>1</v>
       </c>
-      <c r="Z14" s="19">
+      <c r="Z14" s="18">
         <v>2</v>
       </c>
-      <c r="AA14" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="40">
+      <c r="AA14" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="37">
         <f t="shared" si="4"/>
         <v>-9.8520000000000039</v>
       </c>
-      <c r="AC14" s="40">
+      <c r="AC14" s="37">
         <f t="shared" si="5"/>
         <v>-12.799999999999983</v>
       </c>
-      <c r="AD14" s="37"/>
+      <c r="AD14" s="34"/>
     </row>
     <row r="15" spans="1:35" ht="15" customHeight="1">
-      <c r="A15" s="14">
+      <c r="A15" s="13">
         <v>13</v>
       </c>
-      <c r="B15" s="51"/>
-      <c r="C15" s="14" t="s">
+      <c r="B15" s="40"/>
+      <c r="C15" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="14"/>
-      <c r="E15" s="21" t="s">
+      <c r="D15" s="13"/>
+      <c r="E15" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="13">
         <v>321</v>
       </c>
-      <c r="G15" s="23">
+      <c r="G15" s="22">
         <f t="shared" si="0"/>
         <v>292.43099999999998</v>
       </c>
-      <c r="H15" s="23">
+      <c r="H15" s="22">
         <f t="shared" si="1"/>
         <v>288.90000000000003</v>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="17">
         <f t="shared" si="2"/>
         <v>285</v>
       </c>
-      <c r="J15" s="32">
+      <c r="J15" s="30">
         <f t="shared" si="3"/>
         <v>0.88785046728971961</v>
       </c>
-      <c r="K15" s="19">
+      <c r="K15" s="18">
         <v>2</v>
       </c>
-      <c r="L15" s="19">
+      <c r="L15" s="18">
         <v>21</v>
       </c>
-      <c r="M15" s="19">
+      <c r="M15" s="18">
         <v>2</v>
       </c>
-      <c r="N15" s="19">
+      <c r="N15" s="18">
         <v>13</v>
       </c>
-      <c r="O15" s="19">
+      <c r="O15" s="18">
         <v>26</v>
       </c>
-      <c r="P15" s="19">
+      <c r="P15" s="18">
         <v>29</v>
       </c>
-      <c r="Q15" s="19">
+      <c r="Q15" s="18">
         <v>25</v>
       </c>
-      <c r="R15" s="19">
+      <c r="R15" s="18">
         <v>31</v>
       </c>
-      <c r="S15" s="19">
+      <c r="S15" s="18">
         <v>31</v>
       </c>
-      <c r="T15" s="19">
+      <c r="T15" s="18">
         <v>15</v>
       </c>
-      <c r="U15" s="19">
+      <c r="U15" s="18">
         <v>29</v>
       </c>
-      <c r="V15" s="19">
+      <c r="V15" s="18">
         <v>31</v>
       </c>
-      <c r="W15" s="19">
+      <c r="W15" s="18">
         <v>5</v>
       </c>
-      <c r="X15" s="19">
+      <c r="X15" s="18">
         <v>19</v>
       </c>
-      <c r="Y15" s="19">
+      <c r="Y15" s="18">
         <v>1</v>
       </c>
-      <c r="Z15" s="19">
+      <c r="Z15" s="18">
         <v>5</v>
       </c>
-      <c r="AA15" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB15" s="40">
+      <c r="AA15" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="37">
         <f t="shared" si="4"/>
         <v>7.4309999999999832</v>
       </c>
-      <c r="AC15" s="40">
+      <c r="AC15" s="37">
         <f t="shared" si="5"/>
         <v>3.9000000000000341</v>
       </c>
-      <c r="AD15" s="37"/>
+      <c r="AD15" s="34"/>
     </row>
     <row r="16" spans="1:35" ht="15" customHeight="1">
-      <c r="A16" s="14">
+      <c r="A16" s="13">
         <v>14</v>
       </c>
-      <c r="B16" s="51"/>
-      <c r="C16" s="14" t="s">
+      <c r="B16" s="40"/>
+      <c r="C16" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="21" t="s">
+      <c r="D16" s="13"/>
+      <c r="E16" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="14">
+      <c r="F16" s="13">
         <v>199</v>
       </c>
-      <c r="G16" s="23">
+      <c r="G16" s="22">
         <f t="shared" si="0"/>
         <v>181.28899999999999</v>
       </c>
-      <c r="H16" s="23">
+      <c r="H16" s="22">
         <f t="shared" si="1"/>
         <v>179.1</v>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="17">
         <f t="shared" si="2"/>
         <v>191</v>
       </c>
-      <c r="J16" s="32">
+      <c r="J16" s="30">
         <f t="shared" si="3"/>
         <v>0.95979899497487442</v>
       </c>
-      <c r="K16" s="19">
+      <c r="K16" s="18">
         <v>2</v>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="18">
         <v>3</v>
       </c>
-      <c r="M16" s="19">
+      <c r="M16" s="18">
         <v>26</v>
       </c>
-      <c r="N16" s="19">
+      <c r="N16" s="18">
         <v>11</v>
       </c>
-      <c r="O16" s="19">
+      <c r="O16" s="18">
         <v>17</v>
       </c>
-      <c r="P16" s="19">
+      <c r="P16" s="18">
         <v>23</v>
       </c>
-      <c r="Q16" s="19">
+      <c r="Q16" s="18">
         <v>6</v>
       </c>
-      <c r="R16" s="19">
+      <c r="R16" s="18">
         <v>17</v>
       </c>
-      <c r="S16" s="19">
+      <c r="S16" s="18">
         <v>26</v>
       </c>
-      <c r="T16" s="19">
+      <c r="T16" s="18">
         <v>19</v>
       </c>
-      <c r="U16" s="19">
+      <c r="U16" s="18">
         <v>6</v>
       </c>
-      <c r="V16" s="19">
+      <c r="V16" s="18">
         <v>30</v>
       </c>
-      <c r="W16" s="19">
+      <c r="W16" s="18">
         <v>1</v>
       </c>
-      <c r="X16" s="19">
+      <c r="X16" s="18">
         <v>1</v>
       </c>
-      <c r="Y16" s="19">
+      <c r="Y16" s="18">
         <v>1</v>
       </c>
-      <c r="Z16" s="19">
+      <c r="Z16" s="18">
         <v>2</v>
       </c>
-      <c r="AA16" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="40">
+      <c r="AA16" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB16" s="37">
         <f t="shared" si="4"/>
         <v>-9.7110000000000127</v>
       </c>
-      <c r="AC16" s="40">
+      <c r="AC16" s="37">
         <f t="shared" si="5"/>
         <v>-11.900000000000006</v>
       </c>
-      <c r="AD16" s="37"/>
+      <c r="AD16" s="34"/>
     </row>
     <row r="17" spans="1:30" ht="15" customHeight="1">
-      <c r="A17" s="14">
+      <c r="A17" s="13">
         <v>15</v>
       </c>
-      <c r="B17" s="51"/>
-      <c r="C17" s="14" t="s">
+      <c r="B17" s="40"/>
+      <c r="C17" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="14"/>
-      <c r="E17" s="21" t="s">
+      <c r="D17" s="13"/>
+      <c r="E17" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="13">
         <v>273</v>
       </c>
-      <c r="G17" s="23">
+      <c r="G17" s="22">
         <f t="shared" si="0"/>
         <v>248.703</v>
       </c>
-      <c r="H17" s="23">
+      <c r="H17" s="22">
         <f t="shared" si="1"/>
         <v>245.70000000000002</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="17">
         <f t="shared" si="2"/>
         <v>249</v>
       </c>
-      <c r="J17" s="32">
+      <c r="J17" s="30">
         <f t="shared" si="3"/>
         <v>0.91208791208791207</v>
       </c>
-      <c r="K17" s="19">
-        <v>0</v>
-      </c>
-      <c r="L17" s="19">
+      <c r="K17" s="18">
+        <v>0</v>
+      </c>
+      <c r="L17" s="18">
         <v>8</v>
       </c>
-      <c r="M17" s="19">
+      <c r="M17" s="18">
         <v>29</v>
       </c>
-      <c r="N17" s="19">
+      <c r="N17" s="18">
         <v>15</v>
       </c>
-      <c r="O17" s="19">
+      <c r="O17" s="18">
         <v>12</v>
       </c>
-      <c r="P17" s="19">
+      <c r="P17" s="18">
         <v>14</v>
       </c>
-      <c r="Q17" s="19">
+      <c r="Q17" s="18">
         <v>25</v>
       </c>
-      <c r="R17" s="19">
+      <c r="R17" s="18">
         <v>21</v>
       </c>
-      <c r="S17" s="19">
+      <c r="S17" s="18">
         <v>32</v>
       </c>
-      <c r="T17" s="19">
+      <c r="T17" s="18">
         <v>11</v>
       </c>
-      <c r="U17" s="19">
+      <c r="U17" s="18">
         <v>28</v>
       </c>
-      <c r="V17" s="19">
+      <c r="V17" s="18">
         <v>10</v>
       </c>
-      <c r="W17" s="19">
+      <c r="W17" s="18">
         <v>6</v>
       </c>
-      <c r="X17" s="19">
+      <c r="X17" s="18">
         <v>30</v>
       </c>
-      <c r="Y17" s="19">
+      <c r="Y17" s="18">
         <v>4</v>
       </c>
-      <c r="Z17" s="19">
+      <c r="Z17" s="18">
         <v>4</v>
       </c>
-      <c r="AA17" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="40">
+      <c r="AA17" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="37">
         <f t="shared" si="4"/>
         <v>-0.29699999999999704</v>
       </c>
-      <c r="AC17" s="40">
+      <c r="AC17" s="37">
         <f t="shared" si="5"/>
         <v>-3.2999999999999829</v>
       </c>
-      <c r="AD17" s="37"/>
+      <c r="AD17" s="34"/>
     </row>
     <row r="18" spans="1:30" ht="15" customHeight="1">
-      <c r="A18" s="14">
+      <c r="A18" s="13">
         <v>16</v>
       </c>
-      <c r="B18" s="51"/>
-      <c r="C18" s="14" t="s">
+      <c r="B18" s="40"/>
+      <c r="C18" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="21" t="s">
+      <c r="D18" s="13"/>
+      <c r="E18" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="13">
         <v>282</v>
       </c>
-      <c r="G18" s="23">
+      <c r="G18" s="22">
         <f t="shared" si="0"/>
         <v>256.90199999999999</v>
       </c>
-      <c r="H18" s="23">
+      <c r="H18" s="22">
         <f t="shared" si="1"/>
         <v>253.8</v>
       </c>
-      <c r="I18" s="18">
+      <c r="I18" s="17">
         <f t="shared" si="2"/>
         <v>226</v>
       </c>
-      <c r="J18" s="32">
+      <c r="J18" s="30">
         <f t="shared" si="3"/>
         <v>0.8014184397163121</v>
       </c>
-      <c r="K18" s="19">
+      <c r="K18" s="18">
         <v>2</v>
       </c>
-      <c r="L18" s="19">
+      <c r="L18" s="18">
         <v>2</v>
       </c>
-      <c r="M18" s="19">
+      <c r="M18" s="18">
         <v>15</v>
       </c>
-      <c r="N18" s="19">
+      <c r="N18" s="18">
         <v>29</v>
       </c>
-      <c r="O18" s="19">
+      <c r="O18" s="18">
         <v>10</v>
       </c>
-      <c r="P18" s="19">
+      <c r="P18" s="18">
         <v>30</v>
       </c>
-      <c r="Q18" s="19">
+      <c r="Q18" s="18">
         <v>29</v>
       </c>
-      <c r="R18" s="19">
+      <c r="R18" s="18">
         <v>29</v>
       </c>
-      <c r="S18" s="19">
-        <v>0</v>
-      </c>
-      <c r="T18" s="19">
+      <c r="S18" s="18">
+        <v>0</v>
+      </c>
+      <c r="T18" s="18">
         <v>9</v>
       </c>
-      <c r="U18" s="19">
+      <c r="U18" s="18">
         <v>19</v>
       </c>
-      <c r="V18" s="19">
-        <v>0</v>
-      </c>
-      <c r="W18" s="19">
+      <c r="V18" s="18">
+        <v>0</v>
+      </c>
+      <c r="W18" s="18">
         <v>29</v>
       </c>
-      <c r="X18" s="19">
+      <c r="X18" s="18">
         <v>13</v>
       </c>
-      <c r="Y18" s="19">
+      <c r="Y18" s="18">
         <v>5</v>
       </c>
-      <c r="Z18" s="19">
+      <c r="Z18" s="18">
         <v>5</v>
       </c>
-      <c r="AA18" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB18" s="40">
+      <c r="AA18" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="37">
         <f t="shared" si="4"/>
         <v>30.901999999999987</v>
       </c>
-      <c r="AC18" s="40">
+      <c r="AC18" s="37">
         <f t="shared" si="5"/>
         <v>27.800000000000011</v>
       </c>
-      <c r="AD18" s="37"/>
+      <c r="AD18" s="34"/>
     </row>
     <row r="19" spans="1:30" ht="15" customHeight="1">
-      <c r="A19" s="14">
+      <c r="A19" s="13">
         <v>17</v>
       </c>
-      <c r="B19" s="51"/>
-      <c r="C19" s="14" t="s">
+      <c r="B19" s="40"/>
+      <c r="C19" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="14"/>
-      <c r="E19" s="21" t="s">
+      <c r="D19" s="13"/>
+      <c r="E19" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="F19" s="14">
+      <c r="F19" s="13">
         <v>238</v>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="22">
         <f t="shared" si="0"/>
         <v>216.81800000000001</v>
       </c>
-      <c r="H19" s="23">
+      <c r="H19" s="22">
         <f t="shared" si="1"/>
         <v>214.20000000000002</v>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="17">
         <f t="shared" si="2"/>
         <v>204</v>
       </c>
-      <c r="J19" s="32">
+      <c r="J19" s="30">
         <f t="shared" si="3"/>
         <v>0.8571428571428571</v>
       </c>
-      <c r="K19" s="19">
-        <v>0</v>
-      </c>
-      <c r="L19" s="19">
+      <c r="K19" s="18">
+        <v>0</v>
+      </c>
+      <c r="L19" s="18">
         <v>31</v>
       </c>
-      <c r="M19" s="19">
+      <c r="M19" s="18">
         <v>24</v>
       </c>
-      <c r="N19" s="19">
+      <c r="N19" s="18">
         <v>1</v>
       </c>
-      <c r="O19" s="19">
+      <c r="O19" s="18">
         <v>11</v>
       </c>
-      <c r="P19" s="19">
+      <c r="P19" s="18">
         <v>21</v>
       </c>
-      <c r="Q19" s="19">
+      <c r="Q19" s="18">
         <v>1</v>
       </c>
-      <c r="R19" s="19">
+      <c r="R19" s="18">
         <v>22</v>
       </c>
-      <c r="S19" s="19">
+      <c r="S19" s="18">
         <v>17</v>
       </c>
-      <c r="T19" s="19">
+      <c r="T19" s="18">
         <v>12</v>
       </c>
-      <c r="U19" s="19">
+      <c r="U19" s="18">
         <v>11</v>
       </c>
-      <c r="V19" s="19">
+      <c r="V19" s="18">
         <v>7</v>
       </c>
-      <c r="W19" s="19">
+      <c r="W19" s="18">
         <v>19</v>
       </c>
-      <c r="X19" s="19">
+      <c r="X19" s="18">
         <v>21</v>
       </c>
-      <c r="Y19" s="19">
+      <c r="Y19" s="18">
         <v>4</v>
       </c>
-      <c r="Z19" s="19">
+      <c r="Z19" s="18">
         <v>2</v>
       </c>
-      <c r="AA19" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="40">
+      <c r="AA19" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="37">
         <f t="shared" si="4"/>
         <v>12.818000000000012</v>
       </c>
-      <c r="AC19" s="40">
+      <c r="AC19" s="37">
         <f t="shared" si="5"/>
         <v>10.200000000000017</v>
       </c>
-      <c r="AD19" s="37"/>
+      <c r="AD19" s="34"/>
     </row>
     <row r="20" spans="1:30" ht="16.899999999999999" customHeight="1">
-      <c r="A20" s="14">
+      <c r="A20" s="13">
         <v>18</v>
       </c>
-      <c r="B20" s="51"/>
-      <c r="C20" s="14" t="s">
+      <c r="B20" s="40"/>
+      <c r="C20" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="14"/>
-      <c r="E20" s="21" t="s">
+      <c r="D20" s="13"/>
+      <c r="E20" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="13">
         <v>194</v>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="22">
         <f t="shared" si="0"/>
         <v>176.73400000000001</v>
       </c>
-      <c r="H20" s="23">
+      <c r="H20" s="22">
         <f t="shared" si="1"/>
         <v>174.6</v>
       </c>
-      <c r="I20" s="18">
+      <c r="I20" s="17">
         <f t="shared" si="2"/>
         <v>185</v>
       </c>
-      <c r="J20" s="32">
+      <c r="J20" s="30">
         <f t="shared" si="3"/>
         <v>0.95360824742268047</v>
       </c>
-      <c r="K20" s="19">
-        <v>0</v>
-      </c>
-      <c r="L20" s="19">
+      <c r="K20" s="18">
+        <v>0</v>
+      </c>
+      <c r="L20" s="18">
         <v>4</v>
       </c>
-      <c r="M20" s="19">
+      <c r="M20" s="18">
         <v>27</v>
       </c>
-      <c r="N20" s="19">
+      <c r="N20" s="18">
         <v>9</v>
       </c>
-      <c r="O20" s="19">
+      <c r="O20" s="18">
         <v>32</v>
       </c>
-      <c r="P20" s="19">
+      <c r="P20" s="18">
         <v>11</v>
       </c>
-      <c r="Q20" s="19">
-        <v>0</v>
-      </c>
-      <c r="R20" s="19">
+      <c r="Q20" s="18">
+        <v>0</v>
+      </c>
+      <c r="R20" s="18">
         <v>19</v>
       </c>
-      <c r="S20" s="19">
+      <c r="S20" s="18">
         <v>11</v>
       </c>
-      <c r="T20" s="19">
+      <c r="T20" s="18">
         <v>5</v>
       </c>
-      <c r="U20" s="19">
+      <c r="U20" s="18">
         <v>6</v>
       </c>
-      <c r="V20" s="19">
+      <c r="V20" s="18">
         <v>21</v>
       </c>
-      <c r="W20" s="19">
+      <c r="W20" s="18">
         <v>3</v>
       </c>
-      <c r="X20" s="19">
+      <c r="X20" s="18">
         <v>31</v>
       </c>
-      <c r="Y20" s="19">
+      <c r="Y20" s="18">
         <v>1</v>
       </c>
-      <c r="Z20" s="19">
+      <c r="Z20" s="18">
         <v>5</v>
       </c>
-      <c r="AA20" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="40">
+      <c r="AA20" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="37">
         <f t="shared" si="4"/>
         <v>-8.2659999999999911</v>
       </c>
-      <c r="AC20" s="40">
+      <c r="AC20" s="37">
         <f t="shared" si="5"/>
         <v>-10.400000000000006</v>
       </c>
-      <c r="AD20" s="37"/>
+      <c r="AD20" s="34"/>
     </row>
     <row r="21" spans="1:30" ht="15" customHeight="1">
-      <c r="A21" s="14">
+      <c r="A21" s="13">
         <v>19</v>
       </c>
-      <c r="B21" s="51"/>
-      <c r="C21" s="14" t="s">
+      <c r="B21" s="40"/>
+      <c r="C21" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D21" s="14"/>
-      <c r="E21" s="21" t="s">
+      <c r="D21" s="13"/>
+      <c r="E21" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="14">
+      <c r="F21" s="13">
         <v>256</v>
       </c>
-      <c r="G21" s="23">
+      <c r="G21" s="22">
         <f t="shared" si="0"/>
         <v>233.21600000000001</v>
       </c>
-      <c r="H21" s="23">
+      <c r="H21" s="22">
         <f t="shared" si="1"/>
         <v>230.4</v>
       </c>
-      <c r="I21" s="18">
+      <c r="I21" s="17">
         <f t="shared" si="2"/>
         <v>243</v>
       </c>
-      <c r="J21" s="32">
+      <c r="J21" s="30">
         <f t="shared" si="3"/>
         <v>0.94921875</v>
       </c>
-      <c r="K21" s="19">
+      <c r="K21" s="18">
         <v>1</v>
       </c>
-      <c r="L21" s="19">
+      <c r="L21" s="18">
         <v>21</v>
       </c>
-      <c r="M21" s="19">
+      <c r="M21" s="18">
         <v>28</v>
       </c>
-      <c r="N21" s="19">
+      <c r="N21" s="18">
         <v>11</v>
       </c>
-      <c r="O21" s="19">
+      <c r="O21" s="18">
         <v>20</v>
       </c>
-      <c r="P21" s="19">
+      <c r="P21" s="18">
         <v>13</v>
       </c>
-      <c r="Q21" s="19">
+      <c r="Q21" s="18">
         <v>14</v>
       </c>
-      <c r="R21" s="19">
+      <c r="R21" s="18">
         <v>6</v>
       </c>
-      <c r="S21" s="19">
+      <c r="S21" s="18">
         <v>26</v>
       </c>
-      <c r="T21" s="19">
+      <c r="T21" s="18">
         <v>18</v>
       </c>
-      <c r="U21" s="19">
+      <c r="U21" s="18">
         <v>17</v>
       </c>
-      <c r="V21" s="19">
+      <c r="V21" s="18">
         <v>22</v>
       </c>
-      <c r="W21" s="19">
+      <c r="W21" s="18">
         <v>13</v>
       </c>
-      <c r="X21" s="19">
+      <c r="X21" s="18">
         <v>21</v>
       </c>
-      <c r="Y21" s="19">
+      <c r="Y21" s="18">
         <v>7</v>
       </c>
-      <c r="Z21" s="19">
+      <c r="Z21" s="18">
         <v>5</v>
       </c>
-      <c r="AA21" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="40">
+      <c r="AA21" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="37">
         <f t="shared" si="4"/>
         <v>-9.7839999999999918</v>
       </c>
-      <c r="AC21" s="40">
+      <c r="AC21" s="37">
         <f t="shared" si="5"/>
         <v>-12.599999999999994</v>
       </c>
-      <c r="AD21" s="37"/>
+      <c r="AD21" s="34"/>
     </row>
     <row r="22" spans="1:30" ht="15" customHeight="1">
-      <c r="A22" s="14">
+      <c r="A22" s="13">
         <v>20</v>
       </c>
-      <c r="B22" s="51"/>
-      <c r="C22" s="14" t="s">
+      <c r="B22" s="40"/>
+      <c r="C22" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="21" t="s">
+      <c r="D22" s="13"/>
+      <c r="E22" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="F22" s="14">
+      <c r="F22" s="13">
         <v>264</v>
       </c>
-      <c r="G22" s="23">
+      <c r="G22" s="22">
         <f t="shared" si="0"/>
         <v>240.50399999999999</v>
       </c>
-      <c r="H22" s="23">
+      <c r="H22" s="22">
         <f t="shared" si="1"/>
         <v>237.6</v>
       </c>
-      <c r="I22" s="18">
+      <c r="I22" s="17">
         <f t="shared" si="2"/>
         <v>240</v>
       </c>
-      <c r="J22" s="32">
+      <c r="J22" s="30">
         <f t="shared" si="3"/>
         <v>0.90909090909090906</v>
       </c>
-      <c r="K22" s="19">
-        <v>0</v>
-      </c>
-      <c r="L22" s="19">
+      <c r="K22" s="18">
+        <v>0</v>
+      </c>
+      <c r="L22" s="18">
         <v>17</v>
       </c>
-      <c r="M22" s="19">
+      <c r="M22" s="18">
         <v>26</v>
       </c>
-      <c r="N22" s="19">
+      <c r="N22" s="18">
         <v>22</v>
       </c>
-      <c r="O22" s="19">
+      <c r="O22" s="18">
         <v>10</v>
       </c>
-      <c r="P22" s="19">
+      <c r="P22" s="18">
         <v>19</v>
       </c>
-      <c r="Q22" s="19">
+      <c r="Q22" s="18">
         <v>24</v>
       </c>
-      <c r="R22" s="19">
+      <c r="R22" s="18">
         <v>14</v>
       </c>
-      <c r="S22" s="19">
+      <c r="S22" s="18">
         <v>32</v>
       </c>
-      <c r="T22" s="19">
+      <c r="T22" s="18">
         <v>16</v>
       </c>
-      <c r="U22" s="19">
+      <c r="U22" s="18">
         <v>28</v>
       </c>
-      <c r="V22" s="19">
+      <c r="V22" s="18">
         <v>1</v>
       </c>
-      <c r="W22" s="19">
+      <c r="W22" s="18">
         <v>13</v>
       </c>
-      <c r="X22" s="19">
+      <c r="X22" s="18">
         <v>13</v>
       </c>
-      <c r="Y22" s="19">
+      <c r="Y22" s="18">
         <v>1</v>
       </c>
-      <c r="Z22" s="19">
+      <c r="Z22" s="18">
         <v>4</v>
       </c>
-      <c r="AA22" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="40">
+      <c r="AA22" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="37">
         <f t="shared" si="4"/>
         <v>0.50399999999999068</v>
       </c>
-      <c r="AC22" s="40">
+      <c r="AC22" s="37">
         <f t="shared" si="5"/>
         <v>-2.4000000000000057</v>
       </c>
-      <c r="AD22" s="37"/>
+      <c r="AD22" s="34"/>
     </row>
     <row r="23" spans="1:30" ht="15" customHeight="1">
-      <c r="A23" s="14">
+      <c r="A23" s="13">
         <v>21</v>
       </c>
-      <c r="B23" s="51"/>
-      <c r="C23" s="14" t="s">
+      <c r="B23" s="40"/>
+      <c r="C23" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="14"/>
-      <c r="E23" s="21" t="s">
+      <c r="D23" s="13"/>
+      <c r="E23" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="14">
+      <c r="F23" s="13">
         <v>294</v>
       </c>
-      <c r="G23" s="23">
+      <c r="G23" s="22">
         <f t="shared" si="0"/>
         <v>267.834</v>
       </c>
-      <c r="H23" s="23">
+      <c r="H23" s="22">
         <f t="shared" si="1"/>
         <v>264.60000000000002</v>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="17">
         <f t="shared" si="2"/>
         <v>241</v>
       </c>
-      <c r="J23" s="32">
+      <c r="J23" s="30">
         <f t="shared" si="3"/>
         <v>0.81972789115646261</v>
       </c>
-      <c r="K23" s="19">
-        <v>0</v>
-      </c>
-      <c r="L23" s="19">
+      <c r="K23" s="18">
+        <v>0</v>
+      </c>
+      <c r="L23" s="18">
         <v>31</v>
       </c>
-      <c r="M23" s="19">
+      <c r="M23" s="18">
         <v>15</v>
       </c>
-      <c r="N23" s="19">
+      <c r="N23" s="18">
         <v>10</v>
       </c>
-      <c r="O23" s="19">
+      <c r="O23" s="18">
         <v>15</v>
       </c>
-      <c r="P23" s="19">
+      <c r="P23" s="18">
         <v>23</v>
       </c>
-      <c r="Q23" s="19">
+      <c r="Q23" s="18">
         <v>13</v>
       </c>
-      <c r="R23" s="19">
+      <c r="R23" s="18">
         <v>3</v>
       </c>
-      <c r="S23" s="19">
+      <c r="S23" s="18">
         <v>6</v>
       </c>
-      <c r="T23" s="19">
+      <c r="T23" s="18">
         <v>26</v>
       </c>
-      <c r="U23" s="19">
+      <c r="U23" s="18">
         <v>15</v>
       </c>
-      <c r="V23" s="19">
+      <c r="V23" s="18">
         <v>29</v>
       </c>
-      <c r="W23" s="19">
+      <c r="W23" s="18">
         <v>31</v>
       </c>
-      <c r="X23" s="19">
+      <c r="X23" s="18">
         <v>16</v>
       </c>
-      <c r="Y23" s="19">
+      <c r="Y23" s="18">
         <v>1</v>
       </c>
-      <c r="Z23" s="19">
+      <c r="Z23" s="18">
         <v>7</v>
       </c>
-      <c r="AA23" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="40">
+      <c r="AA23" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="37">
         <f t="shared" si="4"/>
         <v>26.834000000000003</v>
       </c>
-      <c r="AC23" s="40">
+      <c r="AC23" s="37">
         <f t="shared" si="5"/>
         <v>23.600000000000023</v>
       </c>
-      <c r="AD23" s="37"/>
+      <c r="AD23" s="34"/>
     </row>
     <row r="24" spans="1:30" ht="15" customHeight="1">
-      <c r="A24" s="14">
+      <c r="A24" s="13">
         <v>22</v>
       </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="14" t="s">
+      <c r="B24" s="40"/>
+      <c r="C24" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="21" t="s">
+      <c r="D24" s="13"/>
+      <c r="E24" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F24" s="14">
+      <c r="F24" s="13">
         <v>200</v>
       </c>
-      <c r="G24" s="23">
+      <c r="G24" s="22">
         <f t="shared" si="0"/>
         <v>182.2</v>
       </c>
-      <c r="H24" s="23">
+      <c r="H24" s="22">
         <f t="shared" si="1"/>
         <v>180</v>
       </c>
-      <c r="I24" s="18">
+      <c r="I24" s="17">
         <f t="shared" si="2"/>
         <v>200</v>
       </c>
-      <c r="J24" s="32">
+      <c r="J24" s="30">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="K24" s="19">
+      <c r="K24" s="18">
         <v>1</v>
       </c>
-      <c r="L24" s="19">
+      <c r="L24" s="18">
         <v>21</v>
       </c>
-      <c r="M24" s="19">
+      <c r="M24" s="18">
         <v>27</v>
       </c>
-      <c r="N24" s="19">
+      <c r="N24" s="18">
         <v>16</v>
       </c>
-      <c r="O24" s="19">
+      <c r="O24" s="18">
         <v>10</v>
       </c>
-      <c r="P24" s="19">
+      <c r="P24" s="18">
         <v>2</v>
       </c>
-      <c r="Q24" s="19">
+      <c r="Q24" s="18">
         <v>3</v>
       </c>
-      <c r="R24" s="19">
+      <c r="R24" s="18">
         <v>29</v>
       </c>
-      <c r="S24" s="19">
+      <c r="S24" s="18">
         <v>20</v>
       </c>
-      <c r="T24" s="19">
+      <c r="T24" s="18">
         <v>30</v>
       </c>
-      <c r="U24" s="19">
+      <c r="U24" s="18">
         <v>18</v>
       </c>
-      <c r="V24" s="19">
+      <c r="V24" s="18">
         <v>5</v>
       </c>
-      <c r="W24" s="19">
+      <c r="W24" s="18">
         <v>12</v>
       </c>
-      <c r="X24" s="19">
+      <c r="X24" s="18">
         <v>4</v>
       </c>
-      <c r="Y24" s="19">
+      <c r="Y24" s="18">
         <v>2</v>
       </c>
-      <c r="Z24" s="19">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB24" s="40">
+      <c r="Z24" s="18">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="37">
         <f t="shared" si="4"/>
         <v>-17.800000000000011</v>
       </c>
-      <c r="AC24" s="40">
+      <c r="AC24" s="37">
         <f t="shared" si="5"/>
         <v>-20</v>
       </c>
-      <c r="AD24" s="37"/>
+      <c r="AD24" s="34"/>
     </row>
     <row r="25" spans="1:30" ht="15" customHeight="1">
-      <c r="A25" s="14">
+      <c r="A25" s="13">
         <v>23</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="14" t="s">
+      <c r="B25" s="40"/>
+      <c r="C25" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D25" s="14"/>
-      <c r="E25" s="21" t="s">
+      <c r="D25" s="13"/>
+      <c r="E25" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F25" s="14">
+      <c r="F25" s="13">
         <v>210</v>
       </c>
-      <c r="G25" s="23">
+      <c r="G25" s="22">
         <f t="shared" si="0"/>
         <v>191.31</v>
       </c>
-      <c r="H25" s="23">
+      <c r="H25" s="22">
         <f t="shared" si="1"/>
         <v>189</v>
       </c>
-      <c r="I25" s="18">
+      <c r="I25" s="17">
         <f t="shared" si="2"/>
         <v>186</v>
       </c>
-      <c r="J25" s="32">
+      <c r="J25" s="30">
         <f t="shared" si="3"/>
         <v>0.88571428571428568</v>
       </c>
-      <c r="K25" s="19">
+      <c r="K25" s="18">
         <v>1</v>
       </c>
-      <c r="L25" s="19">
-        <v>0</v>
-      </c>
-      <c r="M25" s="19">
+      <c r="L25" s="18">
+        <v>0</v>
+      </c>
+      <c r="M25" s="18">
         <v>7</v>
       </c>
-      <c r="N25" s="19">
+      <c r="N25" s="18">
         <v>30</v>
       </c>
-      <c r="O25" s="19">
+      <c r="O25" s="18">
         <v>27</v>
       </c>
-      <c r="P25" s="19">
+      <c r="P25" s="18">
         <v>27</v>
       </c>
-      <c r="Q25" s="19">
+      <c r="Q25" s="18">
         <v>13</v>
       </c>
-      <c r="R25" s="19">
+      <c r="R25" s="18">
         <v>19</v>
       </c>
-      <c r="S25" s="19">
+      <c r="S25" s="18">
         <v>4</v>
       </c>
-      <c r="T25" s="19">
+      <c r="T25" s="18">
         <v>26</v>
       </c>
-      <c r="U25" s="19">
+      <c r="U25" s="18">
         <v>9</v>
       </c>
-      <c r="V25" s="19">
+      <c r="V25" s="18">
         <v>17</v>
       </c>
-      <c r="W25" s="19">
+      <c r="W25" s="18">
         <v>1</v>
       </c>
-      <c r="X25" s="19">
-        <v>0</v>
-      </c>
-      <c r="Y25" s="19">
+      <c r="X25" s="18">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="18">
         <v>5</v>
       </c>
-      <c r="Z25" s="19">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB25" s="40">
+      <c r="Z25" s="18">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="37">
         <f t="shared" si="4"/>
         <v>5.3100000000000023</v>
       </c>
-      <c r="AC25" s="40">
+      <c r="AC25" s="37">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="AD25" s="37"/>
+      <c r="AD25" s="34"/>
     </row>
     <row r="26" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A26" s="14">
+      <c r="A26" s="13">
         <v>24</v>
       </c>
-      <c r="B26" s="51"/>
-      <c r="C26" s="14" t="s">
+      <c r="B26" s="40"/>
+      <c r="C26" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="21" t="s">
+      <c r="D26" s="13"/>
+      <c r="E26" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="F26" s="14">
+      <c r="F26" s="13">
         <v>384</v>
       </c>
-      <c r="G26" s="23">
+      <c r="G26" s="22">
         <f t="shared" si="0"/>
         <v>349.82400000000001</v>
       </c>
-      <c r="H26" s="23">
+      <c r="H26" s="22">
         <f t="shared" si="1"/>
         <v>345.6</v>
       </c>
-      <c r="I26" s="18">
+      <c r="I26" s="17">
         <f t="shared" si="2"/>
         <v>311</v>
       </c>
-      <c r="J26" s="32">
+      <c r="J26" s="30">
         <f t="shared" si="3"/>
         <v>0.80989583333333337</v>
       </c>
-      <c r="K26" s="19">
+      <c r="K26" s="18">
         <v>2</v>
       </c>
-      <c r="L26" s="19">
+      <c r="L26" s="18">
         <v>17</v>
       </c>
-      <c r="M26" s="19">
+      <c r="M26" s="18">
         <v>23</v>
       </c>
-      <c r="N26" s="19">
+      <c r="N26" s="18">
         <v>29</v>
       </c>
-      <c r="O26" s="19">
+      <c r="O26" s="18">
         <v>22</v>
       </c>
-      <c r="P26" s="19">
+      <c r="P26" s="18">
         <v>29</v>
       </c>
-      <c r="Q26" s="19">
+      <c r="Q26" s="18">
         <v>11</v>
       </c>
-      <c r="R26" s="19">
+      <c r="R26" s="18">
         <v>13</v>
       </c>
-      <c r="S26" s="19">
+      <c r="S26" s="18">
         <v>28</v>
       </c>
-      <c r="T26" s="19">
+      <c r="T26" s="18">
         <v>26</v>
       </c>
-      <c r="U26" s="19">
+      <c r="U26" s="18">
         <v>27</v>
       </c>
-      <c r="V26" s="19">
+      <c r="V26" s="18">
         <v>31</v>
       </c>
-      <c r="W26" s="19">
+      <c r="W26" s="18">
         <v>26</v>
       </c>
-      <c r="X26" s="19">
+      <c r="X26" s="18">
         <v>21</v>
       </c>
-      <c r="Y26" s="19">
-        <v>0</v>
-      </c>
-      <c r="Z26" s="19">
+      <c r="Y26" s="18">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="18">
         <v>6</v>
       </c>
-      <c r="AA26" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB26" s="40">
+      <c r="AA26" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="37">
         <f t="shared" si="4"/>
         <v>38.824000000000012</v>
       </c>
-      <c r="AC26" s="40">
+      <c r="AC26" s="37">
         <f t="shared" si="5"/>
         <v>34.600000000000023</v>
       </c>
-      <c r="AD26" s="37"/>
+      <c r="AD26" s="34"/>
     </row>
     <row r="27" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A27" s="14">
+      <c r="A27" s="13">
         <v>25</v>
       </c>
-      <c r="B27" s="51"/>
-      <c r="C27" s="14" t="s">
+      <c r="B27" s="40"/>
+      <c r="C27" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="21" t="s">
+      <c r="D27" s="13"/>
+      <c r="E27" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="F27" s="14">
+      <c r="F27" s="13">
         <v>320</v>
       </c>
-      <c r="G27" s="23">
+      <c r="G27" s="22">
         <f t="shared" si="0"/>
         <v>291.52</v>
       </c>
-      <c r="H27" s="23">
+      <c r="H27" s="22">
         <f t="shared" si="1"/>
         <v>288</v>
       </c>
-      <c r="I27" s="18">
+      <c r="I27" s="17">
         <f t="shared" si="2"/>
         <v>264</v>
       </c>
-      <c r="J27" s="32">
+      <c r="J27" s="30">
         <f t="shared" si="3"/>
         <v>0.82499999999999996</v>
       </c>
-      <c r="K27" s="19">
+      <c r="K27" s="18">
         <v>2</v>
       </c>
-      <c r="L27" s="19">
+      <c r="L27" s="18">
         <v>6</v>
       </c>
-      <c r="M27" s="19">
+      <c r="M27" s="18">
         <v>23</v>
       </c>
-      <c r="N27" s="19">
+      <c r="N27" s="18">
         <v>31</v>
       </c>
-      <c r="O27" s="19">
+      <c r="O27" s="18">
         <v>26</v>
       </c>
-      <c r="P27" s="19">
+      <c r="P27" s="18">
         <v>26</v>
       </c>
-      <c r="Q27" s="19">
+      <c r="Q27" s="18">
         <v>14</v>
       </c>
-      <c r="R27" s="19">
+      <c r="R27" s="18">
         <v>29</v>
       </c>
-      <c r="S27" s="19">
+      <c r="S27" s="18">
         <v>6</v>
       </c>
-      <c r="T27" s="19">
+      <c r="T27" s="18">
         <v>8</v>
       </c>
-      <c r="U27" s="19">
+      <c r="U27" s="18">
         <v>27</v>
       </c>
-      <c r="V27" s="19">
+      <c r="V27" s="18">
         <v>11</v>
       </c>
-      <c r="W27" s="19">
+      <c r="W27" s="18">
         <v>18</v>
       </c>
-      <c r="X27" s="19">
+      <c r="X27" s="18">
         <v>30</v>
       </c>
-      <c r="Y27" s="19">
+      <c r="Y27" s="18">
         <v>7</v>
       </c>
-      <c r="Z27" s="19">
-        <v>0</v>
-      </c>
-      <c r="AA27" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB27" s="40">
+      <c r="Z27" s="18">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="37">
         <f t="shared" si="4"/>
         <v>27.519999999999982</v>
       </c>
-      <c r="AC27" s="40">
+      <c r="AC27" s="37">
         <f t="shared" si="5"/>
         <v>24</v>
       </c>
-      <c r="AD27" s="37"/>
+      <c r="AD27" s="34"/>
     </row>
     <row r="28" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A28" s="14">
+      <c r="A28" s="13">
         <v>26</v>
       </c>
-      <c r="B28" s="51"/>
-      <c r="C28" s="14" t="s">
+      <c r="B28" s="40"/>
+      <c r="C28" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="21" t="s">
+      <c r="D28" s="13"/>
+      <c r="E28" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="F28" s="14">
+      <c r="F28" s="13">
         <v>222</v>
       </c>
-      <c r="G28" s="23">
+      <c r="G28" s="22">
         <f t="shared" si="0"/>
         <v>202.24199999999999</v>
       </c>
-      <c r="H28" s="23">
+      <c r="H28" s="22">
         <f>F28*90%</f>
         <v>199.8</v>
       </c>
-      <c r="I28" s="18">
+      <c r="I28" s="17">
         <f>SUM(K28:AA28)</f>
         <v>216</v>
       </c>
-      <c r="J28" s="32">
+      <c r="J28" s="30">
         <f>I28/F28</f>
         <v>0.97297297297297303</v>
       </c>
-      <c r="K28" s="19">
+      <c r="K28" s="18">
         <v>1</v>
       </c>
-      <c r="L28" s="19">
+      <c r="L28" s="18">
         <v>28</v>
       </c>
-      <c r="M28" s="19">
+      <c r="M28" s="18">
         <v>12</v>
       </c>
-      <c r="N28" s="19">
+      <c r="N28" s="18">
         <v>3</v>
       </c>
-      <c r="O28" s="19">
+      <c r="O28" s="18">
         <v>32</v>
       </c>
-      <c r="P28" s="19">
+      <c r="P28" s="18">
         <v>4</v>
       </c>
-      <c r="Q28" s="19">
+      <c r="Q28" s="18">
         <v>29</v>
       </c>
-      <c r="R28" s="19">
+      <c r="R28" s="18">
         <v>16</v>
       </c>
-      <c r="S28" s="19">
+      <c r="S28" s="18">
         <v>31</v>
       </c>
-      <c r="T28" s="19">
+      <c r="T28" s="18">
         <v>1</v>
       </c>
-      <c r="U28" s="19">
+      <c r="U28" s="18">
         <v>18</v>
       </c>
-      <c r="V28" s="19">
+      <c r="V28" s="18">
         <v>21</v>
       </c>
-      <c r="W28" s="19">
+      <c r="W28" s="18">
         <v>10</v>
       </c>
-      <c r="X28" s="19">
+      <c r="X28" s="18">
         <v>4</v>
       </c>
-      <c r="Y28" s="19">
+      <c r="Y28" s="18">
         <v>1</v>
       </c>
-      <c r="Z28" s="19">
+      <c r="Z28" s="18">
         <v>5</v>
       </c>
-      <c r="AA28" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB28" s="40">
+      <c r="AA28" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="37">
         <f t="shared" si="4"/>
         <v>-13.75800000000001</v>
       </c>
-      <c r="AC28" s="40">
+      <c r="AC28" s="37">
         <f t="shared" si="5"/>
         <v>-16.199999999999989</v>
       </c>
-      <c r="AD28" s="37"/>
+      <c r="AD28" s="34"/>
     </row>
     <row r="29" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A29" s="14">
+      <c r="A29" s="13">
         <v>27</v>
       </c>
-      <c r="B29" s="51"/>
-      <c r="C29" s="14" t="s">
+      <c r="B29" s="40"/>
+      <c r="C29" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D29" s="14"/>
-      <c r="E29" s="21" t="s">
+      <c r="D29" s="13"/>
+      <c r="E29" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="F29" s="14">
+      <c r="F29" s="13">
         <v>304</v>
       </c>
-      <c r="G29" s="23">
+      <c r="G29" s="22">
         <f t="shared" si="0"/>
         <v>276.94400000000002</v>
       </c>
-      <c r="H29" s="23">
+      <c r="H29" s="22">
         <f>F29*90%</f>
         <v>273.60000000000002</v>
       </c>
-      <c r="I29" s="18">
+      <c r="I29" s="17">
         <f>SUM(K29:AA29)</f>
         <v>245</v>
       </c>
-      <c r="J29" s="32">
+      <c r="J29" s="30">
         <f>I29/F29</f>
         <v>0.80592105263157898</v>
       </c>
-      <c r="K29" s="19">
-        <v>0</v>
-      </c>
-      <c r="L29" s="19">
+      <c r="K29" s="18">
+        <v>0</v>
+      </c>
+      <c r="L29" s="18">
         <v>15</v>
       </c>
-      <c r="M29" s="19">
+      <c r="M29" s="18">
         <v>12</v>
       </c>
-      <c r="N29" s="19">
+      <c r="N29" s="18">
         <v>18</v>
       </c>
-      <c r="O29" s="19">
+      <c r="O29" s="18">
         <v>32</v>
       </c>
-      <c r="P29" s="19">
+      <c r="P29" s="18">
         <v>23</v>
       </c>
-      <c r="Q29" s="19">
+      <c r="Q29" s="18">
         <v>9</v>
       </c>
-      <c r="R29" s="19">
+      <c r="R29" s="18">
         <v>32</v>
       </c>
-      <c r="S29" s="19">
+      <c r="S29" s="18">
         <v>15</v>
       </c>
-      <c r="T29" s="19">
+      <c r="T29" s="18">
         <v>20</v>
       </c>
-      <c r="U29" s="19">
+      <c r="U29" s="18">
         <v>17</v>
       </c>
-      <c r="V29" s="19">
+      <c r="V29" s="18">
         <v>1</v>
       </c>
-      <c r="W29" s="19">
+      <c r="W29" s="18">
         <v>9</v>
       </c>
-      <c r="X29" s="19">
+      <c r="X29" s="18">
         <v>28</v>
       </c>
-      <c r="Y29" s="19">
+      <c r="Y29" s="18">
         <v>7</v>
       </c>
-      <c r="Z29" s="19">
+      <c r="Z29" s="18">
         <v>7</v>
       </c>
-      <c r="AA29" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB29" s="40"/>
-      <c r="AC29" s="40"/>
-      <c r="AD29" s="37"/>
+      <c r="AA29" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="37"/>
+      <c r="AC29" s="37"/>
+      <c r="AD29" s="34"/>
     </row>
     <row r="30" spans="1:30" ht="15" customHeight="1">
-      <c r="A30" s="14">
+      <c r="A30" s="13">
         <v>28</v>
       </c>
-      <c r="B30" s="51"/>
-      <c r="C30" s="14" t="s">
+      <c r="B30" s="40"/>
+      <c r="C30" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="21" t="s">
+      <c r="D30" s="13"/>
+      <c r="E30" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="F30" s="14">
+      <c r="F30" s="13">
         <v>274</v>
       </c>
-      <c r="G30" s="23">
+      <c r="G30" s="22">
         <f t="shared" si="0"/>
         <v>249.614</v>
       </c>
-      <c r="H30" s="23">
+      <c r="H30" s="22">
         <f>F30*90%</f>
         <v>246.6</v>
       </c>
-      <c r="I30" s="18">
+      <c r="I30" s="17">
         <f>SUM(K30:AA30)</f>
         <v>246</v>
       </c>
-      <c r="J30" s="32">
+      <c r="J30" s="30">
         <f>I30/F30</f>
         <v>0.8978102189781022</v>
       </c>
-      <c r="K30" s="19">
-        <v>0</v>
-      </c>
-      <c r="L30" s="19">
+      <c r="K30" s="18">
+        <v>0</v>
+      </c>
+      <c r="L30" s="18">
         <v>7</v>
       </c>
-      <c r="M30" s="19">
+      <c r="M30" s="18">
         <v>13</v>
       </c>
-      <c r="N30" s="19">
+      <c r="N30" s="18">
         <v>27</v>
       </c>
-      <c r="O30" s="19">
+      <c r="O30" s="18">
         <v>28</v>
       </c>
-      <c r="P30" s="19">
+      <c r="P30" s="18">
         <v>1</v>
       </c>
-      <c r="Q30" s="19">
+      <c r="Q30" s="18">
         <v>27</v>
       </c>
-      <c r="R30" s="19">
+      <c r="R30" s="18">
         <v>14</v>
       </c>
-      <c r="S30" s="19">
+      <c r="S30" s="18">
         <v>27</v>
       </c>
-      <c r="T30" s="19">
+      <c r="T30" s="18">
         <v>25</v>
       </c>
-      <c r="U30" s="19">
+      <c r="U30" s="18">
         <v>29</v>
       </c>
-      <c r="V30" s="19">
+      <c r="V30" s="18">
         <v>8</v>
       </c>
-      <c r="W30" s="19">
+      <c r="W30" s="18">
         <v>28</v>
       </c>
-      <c r="X30" s="19">
+      <c r="X30" s="18">
         <v>4</v>
       </c>
-      <c r="Y30" s="19">
+      <c r="Y30" s="18">
         <v>4</v>
       </c>
-      <c r="Z30" s="19">
+      <c r="Z30" s="18">
         <v>4</v>
       </c>
-      <c r="AA30" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB30" s="40">
+      <c r="AA30" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="37">
         <f t="shared" si="4"/>
         <v>3.6140000000000043</v>
       </c>
-      <c r="AC30" s="40">
+      <c r="AC30" s="37">
         <f t="shared" si="5"/>
         <v>0.59999999999999432</v>
       </c>
-      <c r="AD30" s="37"/>
+      <c r="AD30" s="34"/>
     </row>
     <row r="31" spans="1:30" ht="15" customHeight="1">
-      <c r="A31" s="45" t="s">
+      <c r="A31" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="45"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="15">
+      <c r="B31" s="47"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="47"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="14">
         <f>SUM(F3:F30)</f>
         <v>6888</v>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="14">
         <f>SUM(G3:G30)</f>
         <v>6274.9679999999998</v>
       </c>
-      <c r="H31" s="15">
+      <c r="H31" s="14">
         <f>SUM(H3:H30)</f>
         <v>6199.2000000000016</v>
       </c>
-      <c r="I31" s="18">
+      <c r="I31" s="17">
         <f>SUM(K31:AA31)</f>
         <v>6105</v>
       </c>
-      <c r="J31" s="24">
+      <c r="J31" s="23">
         <f>I31/F31</f>
         <v>0.88632404181184665</v>
       </c>
-      <c r="K31" s="20">
+      <c r="K31" s="19">
         <f t="shared" ref="K31:AA31" si="6">SUM(K3:K30)</f>
         <v>22</v>
       </c>
-      <c r="L31" s="20">
+      <c r="L31" s="19">
         <f t="shared" si="6"/>
         <v>408</v>
       </c>
-      <c r="M31" s="20">
+      <c r="M31" s="19">
         <f t="shared" si="6"/>
         <v>492</v>
       </c>
-      <c r="N31" s="20">
+      <c r="N31" s="19">
         <f t="shared" si="6"/>
         <v>456</v>
       </c>
-      <c r="O31" s="20">
+      <c r="O31" s="19">
         <f t="shared" si="6"/>
         <v>520</v>
       </c>
-      <c r="P31" s="20">
+      <c r="P31" s="19">
         <f t="shared" si="6"/>
         <v>404</v>
       </c>
-      <c r="Q31" s="20">
+      <c r="Q31" s="19">
         <f t="shared" si="6"/>
         <v>437</v>
       </c>
-      <c r="R31" s="20">
+      <c r="R31" s="19">
         <f t="shared" si="6"/>
         <v>486</v>
       </c>
-      <c r="S31" s="20">
+      <c r="S31" s="19">
         <f t="shared" si="6"/>
         <v>491</v>
       </c>
-      <c r="T31" s="20">
+      <c r="T31" s="19">
         <f t="shared" si="6"/>
         <v>446</v>
       </c>
-      <c r="U31" s="20">
+      <c r="U31" s="19">
         <f t="shared" si="6"/>
         <v>471</v>
       </c>
-      <c r="V31" s="20">
+      <c r="V31" s="19">
         <f t="shared" si="6"/>
         <v>415</v>
       </c>
-      <c r="W31" s="20">
+      <c r="W31" s="19">
         <f t="shared" si="6"/>
         <v>443</v>
       </c>
-      <c r="X31" s="20">
+      <c r="X31" s="19">
         <f t="shared" si="6"/>
         <v>429</v>
       </c>
-      <c r="Y31" s="20">
+      <c r="Y31" s="19">
         <f t="shared" si="6"/>
         <v>87</v>
       </c>
-      <c r="Z31" s="20">
+      <c r="Z31" s="19">
         <f t="shared" si="6"/>
         <v>98</v>
       </c>
-      <c r="AA31" s="20">
+      <c r="AA31" s="19">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AB31" s="40">
+      <c r="AB31" s="37">
         <f>G31-I31</f>
         <v>169.96799999999985</v>
       </c>
-      <c r="AC31" s="40">
+      <c r="AC31" s="37">
         <f>H31-I31</f>
         <v>94.200000000001637</v>
       </c>
-      <c r="AD31" s="37"/>
+      <c r="AD31" s="34"/>
     </row>
     <row r="32" spans="1:30" ht="15" customHeight="1">
-      <c r="B32" s="47" t="s">
+      <c r="B32" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="48"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="39" t="s">
+      <c r="C32" s="50"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="25"/>
-      <c r="J32" s="10"/>
-      <c r="L32" s="25"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+      <c r="I32" s="13"/>
+      <c r="J32" s="13"/>
+      <c r="K32" s="13"/>
+      <c r="L32" s="13"/>
     </row>
     <row r="33" spans="4:23" ht="15" customHeight="1">
-      <c r="D33" s="27"/>
-      <c r="E33" s="30" t="s">
+      <c r="D33" s="26"/>
+      <c r="E33" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="J33" s="10"/>
-      <c r="L33" s="25"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="13"/>
+      <c r="L33" s="13"/>
     </row>
     <row r="34" spans="4:23" ht="12.6" customHeight="1">
-      <c r="D34" s="28"/>
-      <c r="E34" s="22" t="s">
+      <c r="D34" s="27"/>
+      <c r="E34" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="F34" s="29"/>
-      <c r="G34" s="29"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="29"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="36"/>
-      <c r="L34" s="36"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="13"/>
+      <c r="H34" s="13"/>
+      <c r="I34" s="13"/>
+      <c r="J34" s="13"/>
+      <c r="K34" s="13"/>
+      <c r="L34" s="13"/>
       <c r="W34" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="35" spans="4:23" ht="15" hidden="1" customHeight="1">
-      <c r="D35" s="26"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="46"/>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46"/>
-      <c r="I35" s="46"/>
-      <c r="J35" s="46"/>
-      <c r="K35" s="46"/>
-      <c r="L35" s="46"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="48"/>
+      <c r="F35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="48"/>
+      <c r="I35" s="48"/>
+      <c r="J35" s="48"/>
+      <c r="K35" s="48"/>
+      <c r="L35" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="E35:L35"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="AD1:AD2"/>
     <mergeCell ref="AB1:AB2"/>
     <mergeCell ref="AC1:AC2"/>
@@ -3942,9 +3942,6 @@
     <mergeCell ref="V1:W1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="E35:L35"/>
-    <mergeCell ref="B32:C32"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="J3:J31">

</xml_diff>

<commit_message>
fix(thoihieu): bo dinh dang va vien vung F32:L34 duoi bang, giu vien hang Tong va o chu thich <80%
- F32:L34 sheet Tong: Clear Formats, khong vien, khong nen (K32:K34 ghi de style nen trang cua cot K).
- Excel boc vien ca o ke ben qua canh chung, nen dat lai vien duoi F31:L31 va 4 canh E34 ("Ty le <80%").
- So tung o sau khi resolve style: chi 21 o F32:L34 doi; hang 31, E34, sheet data, cong thuc, merge giu nguyen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/AutoJMS/FullStack/UI/ThoiHieu/ThoiHieuKpi.template.xlsx
+++ b/src/AutoJMS/FullStack/UI/ThoiHieu/ThoiHieuKpi.template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" showInkAnnotation="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A98ACE5-16BE-4DAA-B39B-63AB23FCED2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A01F252-F014-48A4-80BA-985CD8BF3BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{47AA215E-EE30-4004-800A-4EDF6E1F8BAD}"/>
   </bookViews>
@@ -696,6 +696,18 @@
     <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -722,18 +734,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1036,18 +1036,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="81" customHeight="1">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
       <c r="K1" s="15" t="s">
         <v>0</v>
       </c>
@@ -1082,27 +1082,27 @@
       <c r="U1" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="41">
+      <c r="V1" s="45">
         <f>T1*91%</f>
         <v>6268.08</v>
       </c>
-      <c r="W1" s="42"/>
+      <c r="W1" s="46"/>
       <c r="X1" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="Y1" s="43">
+      <c r="Y1" s="47">
         <f>T1*90%</f>
         <v>6199.2</v>
       </c>
-      <c r="Z1" s="44"/>
-      <c r="AA1" s="45"/>
-      <c r="AB1" s="39" t="s">
+      <c r="Z1" s="48"/>
+      <c r="AA1" s="49"/>
+      <c r="AB1" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="AC1" s="39" t="s">
+      <c r="AC1" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="AD1" s="38"/>
+      <c r="AD1" s="42"/>
     </row>
     <row r="2" spans="1:35" s="7" customFormat="1" ht="77.25" customHeight="1">
       <c r="A2" s="10" t="s">
@@ -1186,9 +1186,9 @@
       <c r="AA2" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="AB2" s="39"/>
-      <c r="AC2" s="39"/>
-      <c r="AD2" s="38"/>
+      <c r="AB2" s="43"/>
+      <c r="AC2" s="43"/>
+      <c r="AD2" s="42"/>
       <c r="AE2"/>
       <c r="AF2"/>
       <c r="AG2"/>
@@ -1199,7 +1199,7 @@
       <c r="A3" s="13">
         <v>1</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>48</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -1293,7 +1293,7 @@
       <c r="A4" s="13">
         <v>2</v>
       </c>
-      <c r="B4" s="40"/>
+      <c r="B4" s="44"/>
       <c r="C4" s="13" t="s">
         <v>46</v>
       </c>
@@ -1385,7 +1385,7 @@
       <c r="A5" s="13">
         <v>3</v>
       </c>
-      <c r="B5" s="40"/>
+      <c r="B5" s="44"/>
       <c r="C5" s="13" t="s">
         <v>46</v>
       </c>
@@ -1477,7 +1477,7 @@
       <c r="A6" s="13">
         <v>4</v>
       </c>
-      <c r="B6" s="40"/>
+      <c r="B6" s="44"/>
       <c r="C6" s="13" t="s">
         <v>46</v>
       </c>
@@ -1569,7 +1569,7 @@
       <c r="A7" s="13">
         <v>5</v>
       </c>
-      <c r="B7" s="40"/>
+      <c r="B7" s="44"/>
       <c r="C7" s="13" t="s">
         <v>46</v>
       </c>
@@ -1661,7 +1661,7 @@
       <c r="A8" s="13">
         <v>6</v>
       </c>
-      <c r="B8" s="40"/>
+      <c r="B8" s="44"/>
       <c r="C8" s="13" t="s">
         <v>46</v>
       </c>
@@ -1753,7 +1753,7 @@
       <c r="A9" s="13">
         <v>7</v>
       </c>
-      <c r="B9" s="40"/>
+      <c r="B9" s="44"/>
       <c r="C9" s="13" t="s">
         <v>46</v>
       </c>
@@ -1845,7 +1845,7 @@
       <c r="A10" s="13">
         <v>8</v>
       </c>
-      <c r="B10" s="40"/>
+      <c r="B10" s="44"/>
       <c r="C10" s="13" t="s">
         <v>46</v>
       </c>
@@ -1937,7 +1937,7 @@
       <c r="A11" s="13">
         <v>9</v>
       </c>
-      <c r="B11" s="40"/>
+      <c r="B11" s="44"/>
       <c r="C11" s="13" t="s">
         <v>46</v>
       </c>
@@ -2029,7 +2029,7 @@
       <c r="A12" s="13">
         <v>10</v>
       </c>
-      <c r="B12" s="40"/>
+      <c r="B12" s="44"/>
       <c r="C12" s="13" t="s">
         <v>46</v>
       </c>
@@ -2121,7 +2121,7 @@
       <c r="A13" s="13">
         <v>11</v>
       </c>
-      <c r="B13" s="40"/>
+      <c r="B13" s="44"/>
       <c r="C13" s="13" t="s">
         <v>46</v>
       </c>
@@ -2213,7 +2213,7 @@
       <c r="A14" s="13">
         <v>12</v>
       </c>
-      <c r="B14" s="40"/>
+      <c r="B14" s="44"/>
       <c r="C14" s="13" t="s">
         <v>46</v>
       </c>
@@ -2305,7 +2305,7 @@
       <c r="A15" s="13">
         <v>13</v>
       </c>
-      <c r="B15" s="40"/>
+      <c r="B15" s="44"/>
       <c r="C15" s="13" t="s">
         <v>46</v>
       </c>
@@ -2397,7 +2397,7 @@
       <c r="A16" s="13">
         <v>14</v>
       </c>
-      <c r="B16" s="40"/>
+      <c r="B16" s="44"/>
       <c r="C16" s="13" t="s">
         <v>46</v>
       </c>
@@ -2489,7 +2489,7 @@
       <c r="A17" s="13">
         <v>15</v>
       </c>
-      <c r="B17" s="40"/>
+      <c r="B17" s="44"/>
       <c r="C17" s="13" t="s">
         <v>46</v>
       </c>
@@ -2581,7 +2581,7 @@
       <c r="A18" s="13">
         <v>16</v>
       </c>
-      <c r="B18" s="40"/>
+      <c r="B18" s="44"/>
       <c r="C18" s="13" t="s">
         <v>46</v>
       </c>
@@ -2673,7 +2673,7 @@
       <c r="A19" s="13">
         <v>17</v>
       </c>
-      <c r="B19" s="40"/>
+      <c r="B19" s="44"/>
       <c r="C19" s="13" t="s">
         <v>46</v>
       </c>
@@ -2765,7 +2765,7 @@
       <c r="A20" s="13">
         <v>18</v>
       </c>
-      <c r="B20" s="40"/>
+      <c r="B20" s="44"/>
       <c r="C20" s="13" t="s">
         <v>46</v>
       </c>
@@ -2857,7 +2857,7 @@
       <c r="A21" s="13">
         <v>19</v>
       </c>
-      <c r="B21" s="40"/>
+      <c r="B21" s="44"/>
       <c r="C21" s="13" t="s">
         <v>46</v>
       </c>
@@ -2949,7 +2949,7 @@
       <c r="A22" s="13">
         <v>20</v>
       </c>
-      <c r="B22" s="40"/>
+      <c r="B22" s="44"/>
       <c r="C22" s="13" t="s">
         <v>46</v>
       </c>
@@ -3041,7 +3041,7 @@
       <c r="A23" s="13">
         <v>21</v>
       </c>
-      <c r="B23" s="40"/>
+      <c r="B23" s="44"/>
       <c r="C23" s="13" t="s">
         <v>46</v>
       </c>
@@ -3133,7 +3133,7 @@
       <c r="A24" s="13">
         <v>22</v>
       </c>
-      <c r="B24" s="40"/>
+      <c r="B24" s="44"/>
       <c r="C24" s="13" t="s">
         <v>46</v>
       </c>
@@ -3225,7 +3225,7 @@
       <c r="A25" s="13">
         <v>23</v>
       </c>
-      <c r="B25" s="40"/>
+      <c r="B25" s="44"/>
       <c r="C25" s="13" t="s">
         <v>46</v>
       </c>
@@ -3317,7 +3317,7 @@
       <c r="A26" s="13">
         <v>24</v>
       </c>
-      <c r="B26" s="40"/>
+      <c r="B26" s="44"/>
       <c r="C26" s="13" t="s">
         <v>46</v>
       </c>
@@ -3409,7 +3409,7 @@
       <c r="A27" s="13">
         <v>25</v>
       </c>
-      <c r="B27" s="40"/>
+      <c r="B27" s="44"/>
       <c r="C27" s="13" t="s">
         <v>46</v>
       </c>
@@ -3501,7 +3501,7 @@
       <c r="A28" s="13">
         <v>26</v>
       </c>
-      <c r="B28" s="40"/>
+      <c r="B28" s="44"/>
       <c r="C28" s="13" t="s">
         <v>46</v>
       </c>
@@ -3593,7 +3593,7 @@
       <c r="A29" s="13">
         <v>27</v>
       </c>
-      <c r="B29" s="40"/>
+      <c r="B29" s="44"/>
       <c r="C29" s="13" t="s">
         <v>46</v>
       </c>
@@ -3679,7 +3679,7 @@
       <c r="A30" s="13">
         <v>28</v>
       </c>
-      <c r="B30" s="40"/>
+      <c r="B30" s="44"/>
       <c r="C30" s="13" t="s">
         <v>46</v>
       </c>
@@ -3768,13 +3768,13 @@
       <c r="AD30" s="34"/>
     </row>
     <row r="31" spans="1:30" ht="15" customHeight="1">
-      <c r="A31" s="47" t="s">
+      <c r="A31" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="47"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="47"/>
-      <c r="E31" s="47"/>
+      <c r="B31" s="38"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
       <c r="F31" s="14">
         <f>SUM(F3:F30)</f>
         <v>6888</v>
@@ -3874,61 +3874,58 @@
       <c r="AD31" s="34"/>
     </row>
     <row r="32" spans="1:30" ht="15" customHeight="1">
-      <c r="B32" s="49" t="s">
+      <c r="B32" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="50"/>
+      <c r="C32" s="41"/>
       <c r="D32" s="35"/>
       <c r="E32" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="13"/>
+      <c r="F32"/>
+      <c r="G32"/>
+      <c r="H32"/>
+      <c r="I32"/>
+      <c r="K32"/>
+      <c r="L32"/>
     </row>
     <row r="33" spans="4:23" ht="15" customHeight="1">
       <c r="D33" s="26"/>
       <c r="E33" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="13"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="H33"/>
+      <c r="I33"/>
+      <c r="K33"/>
+      <c r="L33"/>
     </row>
     <row r="34" spans="4:23" ht="12.6" customHeight="1">
       <c r="D34" s="27"/>
       <c r="E34" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
-      <c r="J34" s="13"/>
-      <c r="K34" s="13"/>
-      <c r="L34" s="13"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="H34"/>
+      <c r="I34"/>
+      <c r="K34"/>
+      <c r="L34"/>
       <c r="W34" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="35" spans="4:23" ht="15" hidden="1" customHeight="1">
       <c r="D35" s="25"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="48"/>
-      <c r="H35" s="48"/>
-      <c r="I35" s="48"/>
-      <c r="J35" s="48"/>
-      <c r="K35" s="48"/>
-      <c r="L35" s="48"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="39"/>
+      <c r="H35" s="39"/>
+      <c r="I35" s="39"/>
+      <c r="J35" s="39"/>
+      <c r="K35" s="39"/>
+      <c r="L35" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
fix(thoihieu): gop ten NFC/to hop khi nhap file, dua so mau ve 0 truoc khi nhap, chan chia 0 o cot ty le
- Read: chuan hoa ten nhan vien ve NFC va gop khong phan biet hoa thuong (file JMS that co cung mot ten
  o hai dang Unicode; pivot cua file Excel goc tach lam hai nen thieu don o cot F)
- File mau: bo so lieu mau, moi o so = 0, ten/giam sat/ma buu cuc de trong, tieu de khong kem ma buu cuc
- Cot J: IF(F=0, 0, I/F) co dau cach sau dau phay (lexer ReoGrid doc "0,0" thanh mot so)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/AutoJMS/FullStack/UI/ThoiHieu/ThoiHieuKpi.template.xlsx
+++ b/src/AutoJMS/FullStack/UI/ThoiHieu/ThoiHieuKpi.template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" showInkAnnotation="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A01F252-F014-48A4-80BA-985CD8BF3BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF83B65D-4FF4-4F21-8FDD-FA10D2644700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{47AA215E-EE30-4004-800A-4EDF6E1F8BAD}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">Hàng mới: </t>
   </si>
@@ -175,97 +175,7 @@
 90%</t>
   </si>
   <si>
-    <t>214A02</t>
-  </si>
-  <si>
-    <t>BẢNG KÝ NHẬN THỜI HIỆU THEO MỐC THỜI GIAN 214A02</t>
-  </si>
-  <si>
-    <t>Giám sát 01</t>
-  </si>
-  <si>
-    <t>Nhân viên 01</t>
-  </si>
-  <si>
-    <t>Nhân viên 02</t>
-  </si>
-  <si>
-    <t>Nhân viên 03</t>
-  </si>
-  <si>
-    <t>Nhân viên 04</t>
-  </si>
-  <si>
-    <t>Nhân viên 05</t>
-  </si>
-  <si>
-    <t>Nhân viên 06</t>
-  </si>
-  <si>
-    <t>Nhân viên 07</t>
-  </si>
-  <si>
-    <t>Nhân viên 08</t>
-  </si>
-  <si>
-    <t>Nhân viên 09</t>
-  </si>
-  <si>
-    <t>Nhân viên 10</t>
-  </si>
-  <si>
-    <t>Nhân viên 11</t>
-  </si>
-  <si>
-    <t>Nhân viên 12</t>
-  </si>
-  <si>
-    <t>Nhân viên 13</t>
-  </si>
-  <si>
-    <t>Nhân viên 14</t>
-  </si>
-  <si>
-    <t>Nhân viên 15</t>
-  </si>
-  <si>
-    <t>Nhân viên 16</t>
-  </si>
-  <si>
-    <t>Nhân viên 17</t>
-  </si>
-  <si>
-    <t>Nhân viên 18</t>
-  </si>
-  <si>
-    <t>Nhân viên 19</t>
-  </si>
-  <si>
-    <t>Nhân viên 20</t>
-  </si>
-  <si>
-    <t>Nhân viên 21</t>
-  </si>
-  <si>
-    <t>Nhân viên 22</t>
-  </si>
-  <si>
-    <t>Nhân viên 23</t>
-  </si>
-  <si>
-    <t>Nhân viên 24</t>
-  </si>
-  <si>
-    <t>Nhân viên 25</t>
-  </si>
-  <si>
-    <t>Nhân viên 26</t>
-  </si>
-  <si>
-    <t>Nhân viên 27</t>
-  </si>
-  <si>
-    <t>Nhân viên 28</t>
+    <t>BẢNG KÝ NHẬN THỜI HIỆU THEO MỐC THỜI GIAN</t>
   </si>
 </sst>
 </file>
@@ -1037,7 +947,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="81" customHeight="1">
       <c r="A1" s="50" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B1" s="50"/>
       <c r="C1" s="50"/>
@@ -1052,39 +962,39 @@
         <v>0</v>
       </c>
       <c r="L1" s="31">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="M1" s="15" t="s">
         <v>1</v>
       </c>
       <c r="N1" s="31">
-        <v>2950</v>
+        <v>0</v>
       </c>
       <c r="O1" s="15" t="s">
         <v>2</v>
       </c>
       <c r="P1" s="29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="R1" s="31">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="S1" s="15" t="s">
         <v>4</v>
       </c>
       <c r="T1" s="32">
         <f>F31</f>
-        <v>6888</v>
+        <v>0</v>
       </c>
       <c r="U1" s="33" t="s">
         <v>5</v>
       </c>
       <c r="V1" s="45">
         <f>T1*91%</f>
-        <v>6268.08</v>
+        <v>0</v>
       </c>
       <c r="W1" s="46"/>
       <c r="X1" s="33" t="s">
@@ -1092,7 +1002,7 @@
       </c>
       <c r="Y1" s="47">
         <f>T1*90%</f>
-        <v>6199.2</v>
+        <v>0</v>
       </c>
       <c r="Z1" s="48"/>
       <c r="AA1" s="49"/>
@@ -1199,93 +1109,87 @@
       <c r="A3" s="13">
         <v>1</v>
       </c>
-      <c r="B3" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="B3" s="44"/>
+      <c r="C3" s="13"/>
       <c r="D3" s="13"/>
-      <c r="E3" s="20" t="s">
-        <v>49</v>
-      </c>
+      <c r="E3" s="20"/>
       <c r="F3" s="13">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="G3" s="22">
         <f t="shared" ref="G3:G30" si="0">F3*911/1000</f>
-        <v>159.42500000000001</v>
+        <v>0</v>
       </c>
       <c r="H3" s="22">
         <f>F3*90%</f>
-        <v>157.5</v>
+        <v>0</v>
       </c>
       <c r="I3" s="17">
         <f>SUM(K3:AA3)</f>
-        <v>155</v>
+        <v>0</v>
       </c>
       <c r="J3" s="30">
-        <f>I3/F3</f>
-        <v>0.88571428571428568</v>
+        <f t="shared" ref="J3:J30" si="1">IF(F3=0, 0, I3/F3)</f>
+        <v>0</v>
       </c>
       <c r="K3" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L3" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M3" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N3" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="O3" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P3" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="R3" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="S3" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T3" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="U3" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="V3" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="W3" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="X3" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA3" s="18">
         <v>0</v>
       </c>
       <c r="AB3" s="37">
         <f>G3-I3</f>
-        <v>4.4250000000000114</v>
+        <v>0</v>
       </c>
       <c r="AC3" s="37">
         <f>H3-I3</f>
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="AD3" s="34"/>
     </row>
@@ -1294,90 +1198,86 @@
         <v>2</v>
       </c>
       <c r="B4" s="44"/>
-      <c r="C4" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="20" t="s">
-        <v>50</v>
-      </c>
+      <c r="E4" s="20"/>
       <c r="F4" s="13">
-        <v>217</v>
+        <v>0</v>
       </c>
       <c r="G4" s="22">
         <f t="shared" si="0"/>
-        <v>197.68700000000001</v>
+        <v>0</v>
       </c>
       <c r="H4" s="22">
-        <f t="shared" ref="H4:H27" si="1">F4*90%</f>
-        <v>195.3</v>
+        <f t="shared" ref="H4:H27" si="2">F4*90%</f>
+        <v>0</v>
       </c>
       <c r="I4" s="17">
-        <f t="shared" ref="I4:I27" si="2">SUM(K4:AA4)</f>
-        <v>215</v>
+        <f t="shared" ref="I4:I27" si="3">SUM(K4:AA4)</f>
+        <v>0</v>
       </c>
       <c r="J4" s="30">
-        <f t="shared" ref="J4:J27" si="3">I4/F4</f>
-        <v>0.99078341013824889</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="K4" s="18">
         <v>0</v>
       </c>
       <c r="L4" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="M4" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="N4" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O4" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P4" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="R4" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="S4" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="T4" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U4" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="V4" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W4" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="X4" s="18">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="18">
         <v>0</v>
       </c>
       <c r="AB4" s="37">
         <f t="shared" ref="AB4:AB30" si="4">G4-I4</f>
-        <v>-17.312999999999988</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="37">
         <f t="shared" ref="AC4:AC30" si="5">H4-I4</f>
-        <v>-19.699999999999989</v>
+        <v>0</v>
       </c>
       <c r="AD4" s="34"/>
     </row>
@@ -1386,90 +1286,86 @@
         <v>3</v>
       </c>
       <c r="B5" s="44"/>
-      <c r="C5" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C5" s="13"/>
       <c r="D5" s="13"/>
-      <c r="E5" s="20" t="s">
-        <v>51</v>
-      </c>
+      <c r="E5" s="20"/>
       <c r="F5" s="13">
-        <v>198</v>
+        <v>0</v>
       </c>
       <c r="G5" s="22">
         <f t="shared" si="0"/>
-        <v>180.37799999999999</v>
+        <v>0</v>
       </c>
       <c r="H5" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J5" s="30">
         <f t="shared" si="1"/>
-        <v>178.20000000000002</v>
-      </c>
-      <c r="I5" s="17">
-        <f t="shared" si="2"/>
-        <v>185</v>
-      </c>
-      <c r="J5" s="30">
-        <f t="shared" si="3"/>
-        <v>0.93434343434343436</v>
+        <v>0</v>
       </c>
       <c r="K5" s="18">
         <v>0</v>
       </c>
       <c r="L5" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="M5" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="N5" s="18">
         <v>0</v>
       </c>
       <c r="O5" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="P5" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="18">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="R5" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="S5" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T5" s="18">
         <v>0</v>
       </c>
       <c r="U5" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V5" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="W5" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="X5" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="18">
         <v>0</v>
       </c>
       <c r="AB5" s="37">
         <f t="shared" si="4"/>
-        <v>-4.6220000000000141</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="37">
         <f t="shared" si="5"/>
-        <v>-6.7999999999999829</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="34"/>
     </row>
@@ -1478,76 +1374,72 @@
         <v>4</v>
       </c>
       <c r="B6" s="44"/>
-      <c r="C6" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C6" s="13"/>
       <c r="D6" s="13"/>
-      <c r="E6" s="20" t="s">
-        <v>52</v>
-      </c>
+      <c r="E6" s="20"/>
       <c r="F6" s="13">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="G6" s="22">
         <f t="shared" si="0"/>
-        <v>134.828</v>
+        <v>0</v>
       </c>
       <c r="H6" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J6" s="30">
         <f t="shared" si="1"/>
-        <v>133.20000000000002</v>
-      </c>
-      <c r="I6" s="17">
-        <f t="shared" si="2"/>
-        <v>133</v>
-      </c>
-      <c r="J6" s="30">
-        <f t="shared" si="3"/>
-        <v>0.89864864864864868</v>
+        <v>0</v>
       </c>
       <c r="K6" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M6" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="O6" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="P6" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="R6" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="S6" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="T6" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U6" s="18">
         <v>0</v>
       </c>
       <c r="V6" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="W6" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="X6" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="18">
         <v>0</v>
@@ -1557,11 +1449,11 @@
       </c>
       <c r="AB6" s="37">
         <f t="shared" si="4"/>
-        <v>1.828000000000003</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="37">
         <f t="shared" si="5"/>
-        <v>0.20000000000001705</v>
+        <v>0</v>
       </c>
       <c r="AD6" s="34"/>
     </row>
@@ -1570,52 +1462,48 @@
         <v>5</v>
       </c>
       <c r="B7" s="44"/>
-      <c r="C7" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="20" t="s">
-        <v>53</v>
-      </c>
+      <c r="E7" s="20"/>
       <c r="F7" s="13">
-        <v>218</v>
+        <v>0</v>
       </c>
       <c r="G7" s="22">
         <f t="shared" si="0"/>
-        <v>198.59800000000001</v>
+        <v>0</v>
       </c>
       <c r="H7" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="30">
         <f t="shared" si="1"/>
-        <v>196.20000000000002</v>
-      </c>
-      <c r="I7" s="17">
-        <f t="shared" si="2"/>
-        <v>189</v>
-      </c>
-      <c r="J7" s="30">
-        <f t="shared" si="3"/>
-        <v>0.8669724770642202</v>
+        <v>0</v>
       </c>
       <c r="K7" s="18">
         <v>0</v>
       </c>
       <c r="L7" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="M7" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="N7" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O7" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="P7" s="18">
         <v>0</v>
       </c>
       <c r="Q7" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="R7" s="18">
         <v>0</v>
@@ -1624,36 +1512,36 @@
         <v>0</v>
       </c>
       <c r="T7" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U7" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="V7" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W7" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="X7" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA7" s="18">
         <v>0</v>
       </c>
       <c r="AB7" s="37">
         <f t="shared" si="4"/>
-        <v>9.5980000000000132</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="37">
         <f t="shared" si="5"/>
-        <v>7.2000000000000171</v>
+        <v>0</v>
       </c>
       <c r="AD7" s="34"/>
     </row>
@@ -1662,90 +1550,86 @@
         <v>6</v>
       </c>
       <c r="B8" s="44"/>
-      <c r="C8" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C8" s="13"/>
       <c r="D8" s="13"/>
-      <c r="E8" s="20" t="s">
-        <v>54</v>
-      </c>
+      <c r="E8" s="20"/>
       <c r="F8" s="13">
-        <v>243</v>
+        <v>0</v>
       </c>
       <c r="G8" s="22">
         <f t="shared" si="0"/>
-        <v>221.37299999999999</v>
+        <v>0</v>
       </c>
       <c r="H8" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J8" s="30">
         <f t="shared" si="1"/>
-        <v>218.70000000000002</v>
-      </c>
-      <c r="I8" s="17">
-        <f t="shared" si="2"/>
-        <v>234</v>
-      </c>
-      <c r="J8" s="30">
-        <f t="shared" si="3"/>
-        <v>0.96296296296296291</v>
+        <v>0</v>
       </c>
       <c r="K8" s="18">
         <v>0</v>
       </c>
       <c r="L8" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M8" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N8" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="O8" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="P8" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="R8" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S8" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="T8" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="U8" s="18">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="V8" s="18">
         <v>0</v>
       </c>
       <c r="W8" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="X8" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="18">
         <v>0</v>
       </c>
       <c r="AB8" s="37">
         <f t="shared" si="4"/>
-        <v>-12.62700000000001</v>
+        <v>0</v>
       </c>
       <c r="AC8" s="37">
         <f t="shared" si="5"/>
-        <v>-15.299999999999983</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="34"/>
     </row>
@@ -1754,90 +1638,86 @@
         <v>7</v>
       </c>
       <c r="B9" s="44"/>
-      <c r="C9" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="20" t="s">
-        <v>55</v>
-      </c>
+      <c r="E9" s="20"/>
       <c r="F9" s="13">
-        <v>257</v>
+        <v>0</v>
       </c>
       <c r="G9" s="22">
         <f t="shared" si="0"/>
-        <v>234.12700000000001</v>
+        <v>0</v>
       </c>
       <c r="H9" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="30">
         <f t="shared" si="1"/>
-        <v>231.3</v>
-      </c>
-      <c r="I9" s="17">
-        <f t="shared" si="2"/>
-        <v>221</v>
-      </c>
-      <c r="J9" s="30">
-        <f t="shared" si="3"/>
-        <v>0.8599221789883269</v>
+        <v>0</v>
       </c>
       <c r="K9" s="18">
         <v>0</v>
       </c>
       <c r="L9" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="M9" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N9" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="O9" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P9" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R9" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="S9" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="T9" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="U9" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="V9" s="18">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="W9" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="X9" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA9" s="18">
         <v>0</v>
       </c>
       <c r="AB9" s="37">
         <f t="shared" si="4"/>
-        <v>13.12700000000001</v>
+        <v>0</v>
       </c>
       <c r="AC9" s="37">
         <f t="shared" si="5"/>
-        <v>10.300000000000011</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="34"/>
     </row>
@@ -1846,90 +1726,86 @@
         <v>8</v>
       </c>
       <c r="B10" s="44"/>
-      <c r="C10" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C10" s="13"/>
       <c r="D10" s="13"/>
-      <c r="E10" s="20" t="s">
-        <v>56</v>
-      </c>
+      <c r="E10" s="20"/>
       <c r="F10" s="13">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="G10" s="22">
         <f t="shared" si="0"/>
-        <v>153.959</v>
+        <v>0</v>
       </c>
       <c r="H10" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I10" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="30">
         <f t="shared" si="1"/>
-        <v>152.1</v>
-      </c>
-      <c r="I10" s="17">
-        <f t="shared" si="2"/>
-        <v>142</v>
-      </c>
-      <c r="J10" s="30">
-        <f t="shared" si="3"/>
-        <v>0.84023668639053251</v>
+        <v>0</v>
       </c>
       <c r="K10" s="18">
         <v>0</v>
       </c>
       <c r="L10" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M10" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N10" s="18">
         <v>0</v>
       </c>
       <c r="O10" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P10" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R10" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S10" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="T10" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="U10" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V10" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="W10" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X10" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z10" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA10" s="18">
         <v>0</v>
       </c>
       <c r="AB10" s="37">
         <f t="shared" si="4"/>
-        <v>11.959000000000003</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="37">
         <f t="shared" si="5"/>
-        <v>10.099999999999994</v>
+        <v>0</v>
       </c>
       <c r="AD10" s="34"/>
     </row>
@@ -1938,76 +1814,72 @@
         <v>9</v>
       </c>
       <c r="B11" s="44"/>
-      <c r="C11" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C11" s="13"/>
       <c r="D11" s="13"/>
-      <c r="E11" s="20" t="s">
-        <v>57</v>
-      </c>
+      <c r="E11" s="20"/>
       <c r="F11" s="13">
-        <v>217</v>
+        <v>0</v>
       </c>
       <c r="G11" s="22">
         <f t="shared" si="0"/>
-        <v>197.68700000000001</v>
+        <v>0</v>
       </c>
       <c r="H11" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I11" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J11" s="30">
         <f t="shared" si="1"/>
-        <v>195.3</v>
-      </c>
-      <c r="I11" s="17">
-        <f t="shared" si="2"/>
-        <v>205</v>
-      </c>
-      <c r="J11" s="30">
-        <f t="shared" si="3"/>
-        <v>0.9447004608294931</v>
+        <v>0</v>
       </c>
       <c r="K11" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L11" s="18">
         <v>0</v>
       </c>
       <c r="M11" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="O11" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="P11" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="R11" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="S11" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T11" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="U11" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="V11" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="W11" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X11" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="18">
         <v>0</v>
@@ -2017,11 +1889,11 @@
       </c>
       <c r="AB11" s="37">
         <f t="shared" si="4"/>
-        <v>-7.3129999999999882</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="37">
         <f t="shared" si="5"/>
-        <v>-9.6999999999999886</v>
+        <v>0</v>
       </c>
       <c r="AD11" s="34"/>
     </row>
@@ -2030,90 +1902,86 @@
         <v>10</v>
       </c>
       <c r="B12" s="44"/>
-      <c r="C12" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C12" s="13"/>
       <c r="D12" s="13"/>
-      <c r="E12" s="20" t="s">
-        <v>58</v>
-      </c>
+      <c r="E12" s="20"/>
       <c r="F12" s="13">
-        <v>292</v>
+        <v>0</v>
       </c>
       <c r="G12" s="22">
         <f t="shared" si="0"/>
-        <v>266.012</v>
+        <v>0</v>
       </c>
       <c r="H12" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I12" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J12" s="30">
         <f t="shared" si="1"/>
-        <v>262.8</v>
-      </c>
-      <c r="I12" s="17">
-        <f t="shared" si="2"/>
-        <v>235</v>
-      </c>
-      <c r="J12" s="30">
-        <f t="shared" si="3"/>
-        <v>0.8047945205479452</v>
+        <v>0</v>
       </c>
       <c r="K12" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L12" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="M12" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="N12" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O12" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="P12" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="R12" s="18">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="S12" s="18">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="T12" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="U12" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V12" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="W12" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="X12" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="18">
         <v>0</v>
       </c>
       <c r="AB12" s="37">
         <f t="shared" si="4"/>
-        <v>31.012</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="37">
         <f t="shared" si="5"/>
-        <v>27.800000000000011</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="34"/>
     </row>
@@ -2122,90 +1990,86 @@
         <v>11</v>
       </c>
       <c r="B13" s="44"/>
-      <c r="C13" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C13" s="13"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="20" t="s">
-        <v>59</v>
-      </c>
+      <c r="E13" s="20"/>
       <c r="F13" s="13">
-        <v>251</v>
+        <v>0</v>
       </c>
       <c r="G13" s="22">
         <f t="shared" si="0"/>
-        <v>228.661</v>
+        <v>0</v>
       </c>
       <c r="H13" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I13" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J13" s="30">
         <f t="shared" si="1"/>
-        <v>225.9</v>
-      </c>
-      <c r="I13" s="17">
-        <f t="shared" si="2"/>
-        <v>205</v>
-      </c>
-      <c r="J13" s="30">
-        <f t="shared" si="3"/>
-        <v>0.81673306772908372</v>
+        <v>0</v>
       </c>
       <c r="K13" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L13" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="M13" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="N13" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="O13" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P13" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="18">
         <v>0</v>
       </c>
       <c r="R13" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S13" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="T13" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="U13" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="V13" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="W13" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="X13" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y13" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA13" s="18">
         <v>0</v>
       </c>
       <c r="AB13" s="37">
         <f t="shared" si="4"/>
-        <v>23.661000000000001</v>
+        <v>0</v>
       </c>
       <c r="AC13" s="37">
         <f t="shared" si="5"/>
-        <v>20.900000000000006</v>
+        <v>0</v>
       </c>
       <c r="AD13" s="34"/>
     </row>
@@ -2214,90 +2078,86 @@
         <v>12</v>
       </c>
       <c r="B14" s="44"/>
-      <c r="C14" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="20" t="s">
-        <v>60</v>
-      </c>
+      <c r="E14" s="20"/>
       <c r="F14" s="13">
-        <v>268</v>
+        <v>0</v>
       </c>
       <c r="G14" s="22">
         <f t="shared" si="0"/>
-        <v>244.148</v>
+        <v>0</v>
       </c>
       <c r="H14" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I14" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J14" s="30">
         <f t="shared" si="1"/>
-        <v>241.20000000000002</v>
-      </c>
-      <c r="I14" s="17">
-        <f t="shared" si="2"/>
-        <v>254</v>
-      </c>
-      <c r="J14" s="30">
-        <f t="shared" si="3"/>
-        <v>0.94776119402985071</v>
+        <v>0</v>
       </c>
       <c r="K14" s="18">
         <v>0</v>
       </c>
       <c r="L14" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M14" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="N14" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="O14" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="P14" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="18">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="R14" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S14" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="T14" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="U14" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V14" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="W14" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="X14" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z14" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA14" s="18">
         <v>0</v>
       </c>
       <c r="AB14" s="37">
         <f t="shared" si="4"/>
-        <v>-9.8520000000000039</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="37">
         <f t="shared" si="5"/>
-        <v>-12.799999999999983</v>
+        <v>0</v>
       </c>
       <c r="AD14" s="34"/>
     </row>
@@ -2306,90 +2166,86 @@
         <v>13</v>
       </c>
       <c r="B15" s="44"/>
-      <c r="C15" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C15" s="13"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="20" t="s">
-        <v>61</v>
-      </c>
+      <c r="E15" s="20"/>
       <c r="F15" s="13">
-        <v>321</v>
+        <v>0</v>
       </c>
       <c r="G15" s="22">
         <f t="shared" si="0"/>
-        <v>292.43099999999998</v>
+        <v>0</v>
       </c>
       <c r="H15" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I15" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J15" s="30">
         <f t="shared" si="1"/>
-        <v>288.90000000000003</v>
-      </c>
-      <c r="I15" s="17">
-        <f t="shared" si="2"/>
-        <v>285</v>
-      </c>
-      <c r="J15" s="30">
-        <f t="shared" si="3"/>
-        <v>0.88785046728971961</v>
+        <v>0</v>
       </c>
       <c r="K15" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L15" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="M15" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N15" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O15" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="P15" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="R15" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="S15" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="T15" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="U15" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="V15" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="W15" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="X15" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="Y15" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z15" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA15" s="18">
         <v>0</v>
       </c>
       <c r="AB15" s="37">
         <f t="shared" si="4"/>
-        <v>7.4309999999999832</v>
+        <v>0</v>
       </c>
       <c r="AC15" s="37">
         <f t="shared" si="5"/>
-        <v>3.9000000000000341</v>
+        <v>0</v>
       </c>
       <c r="AD15" s="34"/>
     </row>
@@ -2398,90 +2254,86 @@
         <v>14</v>
       </c>
       <c r="B16" s="44"/>
-      <c r="C16" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C16" s="13"/>
       <c r="D16" s="13"/>
-      <c r="E16" s="20" t="s">
-        <v>62</v>
-      </c>
+      <c r="E16" s="20"/>
       <c r="F16" s="13">
-        <v>199</v>
+        <v>0</v>
       </c>
       <c r="G16" s="22">
         <f t="shared" si="0"/>
-        <v>181.28899999999999</v>
+        <v>0</v>
       </c>
       <c r="H16" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I16" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J16" s="30">
         <f t="shared" si="1"/>
-        <v>179.1</v>
-      </c>
-      <c r="I16" s="17">
-        <f t="shared" si="2"/>
-        <v>191</v>
-      </c>
-      <c r="J16" s="30">
-        <f t="shared" si="3"/>
-        <v>0.95979899497487442</v>
+        <v>0</v>
       </c>
       <c r="K16" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L16" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M16" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N16" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O16" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="P16" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R16" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="S16" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="T16" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="U16" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V16" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="W16" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X16" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y16" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z16" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA16" s="18">
         <v>0</v>
       </c>
       <c r="AB16" s="37">
         <f t="shared" si="4"/>
-        <v>-9.7110000000000127</v>
+        <v>0</v>
       </c>
       <c r="AC16" s="37">
         <f t="shared" si="5"/>
-        <v>-11.900000000000006</v>
+        <v>0</v>
       </c>
       <c r="AD16" s="34"/>
     </row>
@@ -2490,90 +2342,86 @@
         <v>15</v>
       </c>
       <c r="B17" s="44"/>
-      <c r="C17" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C17" s="13"/>
       <c r="D17" s="13"/>
-      <c r="E17" s="20" t="s">
-        <v>63</v>
-      </c>
+      <c r="E17" s="20"/>
       <c r="F17" s="13">
-        <v>273</v>
+        <v>0</v>
       </c>
       <c r="G17" s="22">
         <f t="shared" si="0"/>
-        <v>248.703</v>
+        <v>0</v>
       </c>
       <c r="H17" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I17" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J17" s="30">
         <f t="shared" si="1"/>
-        <v>245.70000000000002</v>
-      </c>
-      <c r="I17" s="17">
-        <f t="shared" si="2"/>
-        <v>249</v>
-      </c>
-      <c r="J17" s="30">
-        <f t="shared" si="3"/>
-        <v>0.91208791208791207</v>
+        <v>0</v>
       </c>
       <c r="K17" s="18">
         <v>0</v>
       </c>
       <c r="L17" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M17" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="N17" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="O17" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P17" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="R17" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="S17" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="T17" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="U17" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="V17" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="W17" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X17" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Y17" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z17" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA17" s="18">
         <v>0</v>
       </c>
       <c r="AB17" s="37">
         <f t="shared" si="4"/>
-        <v>-0.29699999999999704</v>
+        <v>0</v>
       </c>
       <c r="AC17" s="37">
         <f t="shared" si="5"/>
-        <v>-3.2999999999999829</v>
+        <v>0</v>
       </c>
       <c r="AD17" s="34"/>
     </row>
@@ -2582,90 +2430,86 @@
         <v>16</v>
       </c>
       <c r="B18" s="44"/>
-      <c r="C18" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="20" t="s">
-        <v>64</v>
-      </c>
+      <c r="E18" s="20"/>
       <c r="F18" s="13">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="G18" s="22">
         <f t="shared" si="0"/>
-        <v>256.90199999999999</v>
+        <v>0</v>
       </c>
       <c r="H18" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I18" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="30">
         <f t="shared" si="1"/>
-        <v>253.8</v>
-      </c>
-      <c r="I18" s="17">
-        <f t="shared" si="2"/>
-        <v>226</v>
-      </c>
-      <c r="J18" s="30">
-        <f t="shared" si="3"/>
-        <v>0.8014184397163121</v>
+        <v>0</v>
       </c>
       <c r="K18" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L18" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M18" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="N18" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="O18" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P18" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="R18" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="S18" s="18">
         <v>0</v>
       </c>
       <c r="T18" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U18" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="V18" s="18">
         <v>0</v>
       </c>
       <c r="W18" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="X18" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Y18" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="18">
         <v>0</v>
       </c>
       <c r="AB18" s="37">
         <f t="shared" si="4"/>
-        <v>30.901999999999987</v>
+        <v>0</v>
       </c>
       <c r="AC18" s="37">
         <f t="shared" si="5"/>
-        <v>27.800000000000011</v>
+        <v>0</v>
       </c>
       <c r="AD18" s="34"/>
     </row>
@@ -2674,90 +2518,86 @@
         <v>17</v>
       </c>
       <c r="B19" s="44"/>
-      <c r="C19" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="20" t="s">
-        <v>65</v>
-      </c>
+      <c r="E19" s="20"/>
       <c r="F19" s="13">
-        <v>238</v>
+        <v>0</v>
       </c>
       <c r="G19" s="22">
         <f t="shared" si="0"/>
-        <v>216.81800000000001</v>
+        <v>0</v>
       </c>
       <c r="H19" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I19" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="30">
         <f t="shared" si="1"/>
-        <v>214.20000000000002</v>
-      </c>
-      <c r="I19" s="17">
-        <f t="shared" si="2"/>
-        <v>204</v>
-      </c>
-      <c r="J19" s="30">
-        <f t="shared" si="3"/>
-        <v>0.8571428571428571</v>
+        <v>0</v>
       </c>
       <c r="K19" s="18">
         <v>0</v>
       </c>
       <c r="L19" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="M19" s="18">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="N19" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O19" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="P19" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R19" s="18">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="S19" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="T19" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="U19" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="V19" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="W19" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="X19" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Y19" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="18">
         <v>0</v>
       </c>
       <c r="AB19" s="37">
         <f t="shared" si="4"/>
-        <v>12.818000000000012</v>
+        <v>0</v>
       </c>
       <c r="AC19" s="37">
         <f t="shared" si="5"/>
-        <v>10.200000000000017</v>
+        <v>0</v>
       </c>
       <c r="AD19" s="34"/>
     </row>
@@ -2766,90 +2606,86 @@
         <v>18</v>
       </c>
       <c r="B20" s="44"/>
-      <c r="C20" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="20" t="s">
-        <v>66</v>
-      </c>
+      <c r="E20" s="20"/>
       <c r="F20" s="13">
-        <v>194</v>
+        <v>0</v>
       </c>
       <c r="G20" s="22">
         <f t="shared" si="0"/>
-        <v>176.73400000000001</v>
+        <v>0</v>
       </c>
       <c r="H20" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="30">
         <f t="shared" si="1"/>
-        <v>174.6</v>
-      </c>
-      <c r="I20" s="17">
-        <f t="shared" si="2"/>
-        <v>185</v>
-      </c>
-      <c r="J20" s="30">
-        <f t="shared" si="3"/>
-        <v>0.95360824742268047</v>
+        <v>0</v>
       </c>
       <c r="K20" s="18">
         <v>0</v>
       </c>
       <c r="L20" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M20" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="N20" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O20" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="P20" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="18">
         <v>0</v>
       </c>
       <c r="R20" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="S20" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="T20" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U20" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V20" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W20" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X20" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="Y20" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z20" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA20" s="18">
         <v>0</v>
       </c>
       <c r="AB20" s="37">
         <f t="shared" si="4"/>
-        <v>-8.2659999999999911</v>
+        <v>0</v>
       </c>
       <c r="AC20" s="37">
         <f t="shared" si="5"/>
-        <v>-10.400000000000006</v>
+        <v>0</v>
       </c>
       <c r="AD20" s="34"/>
     </row>
@@ -2858,90 +2694,86 @@
         <v>19</v>
       </c>
       <c r="B21" s="44"/>
-      <c r="C21" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="20" t="s">
-        <v>67</v>
-      </c>
+      <c r="E21" s="20"/>
       <c r="F21" s="13">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="G21" s="22">
         <f t="shared" si="0"/>
-        <v>233.21600000000001</v>
+        <v>0</v>
       </c>
       <c r="H21" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="30">
         <f t="shared" si="1"/>
-        <v>230.4</v>
-      </c>
-      <c r="I21" s="17">
-        <f t="shared" si="2"/>
-        <v>243</v>
-      </c>
-      <c r="J21" s="30">
-        <f t="shared" si="3"/>
-        <v>0.94921875</v>
+        <v>0</v>
       </c>
       <c r="K21" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="M21" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N21" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O21" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P21" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="R21" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S21" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="T21" s="18">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="U21" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="V21" s="18">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="W21" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="X21" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Y21" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z21" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA21" s="18">
         <v>0</v>
       </c>
       <c r="AB21" s="37">
         <f t="shared" si="4"/>
-        <v>-9.7839999999999918</v>
+        <v>0</v>
       </c>
       <c r="AC21" s="37">
         <f t="shared" si="5"/>
-        <v>-12.599999999999994</v>
+        <v>0</v>
       </c>
       <c r="AD21" s="34"/>
     </row>
@@ -2950,90 +2782,86 @@
         <v>20</v>
       </c>
       <c r="B22" s="44"/>
-      <c r="C22" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="20" t="s">
-        <v>68</v>
-      </c>
+      <c r="E22" s="20"/>
       <c r="F22" s="13">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="G22" s="22">
         <f t="shared" si="0"/>
-        <v>240.50399999999999</v>
+        <v>0</v>
       </c>
       <c r="H22" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I22" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J22" s="30">
         <f t="shared" si="1"/>
-        <v>237.6</v>
-      </c>
-      <c r="I22" s="17">
-        <f t="shared" si="2"/>
-        <v>240</v>
-      </c>
-      <c r="J22" s="30">
-        <f t="shared" si="3"/>
-        <v>0.90909090909090906</v>
+        <v>0</v>
       </c>
       <c r="K22" s="18">
         <v>0</v>
       </c>
       <c r="L22" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="M22" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N22" s="18">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="O22" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P22" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="18">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="R22" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="S22" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="T22" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="U22" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="V22" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W22" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="X22" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Y22" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z22" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA22" s="18">
         <v>0</v>
       </c>
       <c r="AB22" s="37">
         <f t="shared" si="4"/>
-        <v>0.50399999999999068</v>
+        <v>0</v>
       </c>
       <c r="AC22" s="37">
         <f t="shared" si="5"/>
-        <v>-2.4000000000000057</v>
+        <v>0</v>
       </c>
       <c r="AD22" s="34"/>
     </row>
@@ -3042,90 +2870,86 @@
         <v>21</v>
       </c>
       <c r="B23" s="44"/>
-      <c r="C23" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C23" s="13"/>
       <c r="D23" s="13"/>
-      <c r="E23" s="20" t="s">
-        <v>69</v>
-      </c>
+      <c r="E23" s="20"/>
       <c r="F23" s="13">
-        <v>294</v>
+        <v>0</v>
       </c>
       <c r="G23" s="22">
         <f t="shared" si="0"/>
-        <v>267.834</v>
+        <v>0</v>
       </c>
       <c r="H23" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I23" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="30">
         <f t="shared" si="1"/>
-        <v>264.60000000000002</v>
-      </c>
-      <c r="I23" s="17">
-        <f t="shared" si="2"/>
-        <v>241</v>
-      </c>
-      <c r="J23" s="30">
-        <f t="shared" si="3"/>
-        <v>0.81972789115646261</v>
+        <v>0</v>
       </c>
       <c r="K23" s="18">
         <v>0</v>
       </c>
       <c r="L23" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="M23" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="N23" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O23" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P23" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q23" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="R23" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S23" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T23" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="U23" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="V23" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="W23" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="X23" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="Y23" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z23" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA23" s="18">
         <v>0</v>
       </c>
       <c r="AB23" s="37">
         <f t="shared" si="4"/>
-        <v>26.834000000000003</v>
+        <v>0</v>
       </c>
       <c r="AC23" s="37">
         <f t="shared" si="5"/>
-        <v>23.600000000000023</v>
+        <v>0</v>
       </c>
       <c r="AD23" s="34"/>
     </row>
@@ -3134,76 +2958,72 @@
         <v>22</v>
       </c>
       <c r="B24" s="44"/>
-      <c r="C24" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="20" t="s">
-        <v>70</v>
-      </c>
+      <c r="E24" s="20"/>
       <c r="F24" s="13">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G24" s="22">
         <f t="shared" si="0"/>
-        <v>182.2</v>
+        <v>0</v>
       </c>
       <c r="H24" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I24" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J24" s="30">
         <f t="shared" si="1"/>
-        <v>180</v>
-      </c>
-      <c r="I24" s="17">
-        <f t="shared" si="2"/>
-        <v>200</v>
-      </c>
-      <c r="J24" s="30">
-        <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="M24" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="N24" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O24" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P24" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R24" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="S24" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="T24" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="U24" s="18">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V24" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W24" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="X24" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y24" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z24" s="18">
         <v>0</v>
@@ -3213,11 +3033,11 @@
       </c>
       <c r="AB24" s="37">
         <f t="shared" si="4"/>
-        <v>-17.800000000000011</v>
+        <v>0</v>
       </c>
       <c r="AC24" s="37">
         <f t="shared" si="5"/>
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="AD24" s="34"/>
     </row>
@@ -3226,76 +3046,72 @@
         <v>23</v>
       </c>
       <c r="B25" s="44"/>
-      <c r="C25" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="20" t="s">
-        <v>71</v>
-      </c>
+      <c r="E25" s="20"/>
       <c r="F25" s="13">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="G25" s="22">
         <f t="shared" si="0"/>
-        <v>191.31</v>
+        <v>0</v>
       </c>
       <c r="H25" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I25" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J25" s="30">
         <f t="shared" si="1"/>
-        <v>189</v>
-      </c>
-      <c r="I25" s="17">
-        <f t="shared" si="2"/>
-        <v>186</v>
-      </c>
-      <c r="J25" s="30">
-        <f t="shared" si="3"/>
-        <v>0.88571428571428568</v>
+        <v>0</v>
       </c>
       <c r="K25" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L25" s="18">
         <v>0</v>
       </c>
       <c r="M25" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N25" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="O25" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="P25" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="R25" s="18">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="S25" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T25" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="U25" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V25" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="W25" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X25" s="18">
         <v>0</v>
       </c>
       <c r="Y25" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Z25" s="18">
         <v>0</v>
@@ -3305,11 +3121,11 @@
       </c>
       <c r="AB25" s="37">
         <f t="shared" si="4"/>
-        <v>5.3100000000000023</v>
+        <v>0</v>
       </c>
       <c r="AC25" s="37">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD25" s="34"/>
     </row>
@@ -3318,90 +3134,86 @@
         <v>24</v>
       </c>
       <c r="B26" s="44"/>
-      <c r="C26" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C26" s="13"/>
       <c r="D26" s="13"/>
-      <c r="E26" s="20" t="s">
-        <v>72</v>
-      </c>
+      <c r="E26" s="20"/>
       <c r="F26" s="13">
-        <v>384</v>
+        <v>0</v>
       </c>
       <c r="G26" s="22">
         <f t="shared" si="0"/>
-        <v>349.82400000000001</v>
+        <v>0</v>
       </c>
       <c r="H26" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I26" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J26" s="30">
         <f t="shared" si="1"/>
-        <v>345.6</v>
-      </c>
-      <c r="I26" s="17">
-        <f t="shared" si="2"/>
-        <v>311</v>
-      </c>
-      <c r="J26" s="30">
-        <f t="shared" si="3"/>
-        <v>0.80989583333333337</v>
+        <v>0</v>
       </c>
       <c r="K26" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L26" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="M26" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="N26" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="O26" s="18">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="P26" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="Q26" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="R26" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S26" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="T26" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="U26" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="V26" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="W26" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="X26" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Y26" s="18">
         <v>0</v>
       </c>
       <c r="Z26" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA26" s="18">
         <v>0</v>
       </c>
       <c r="AB26" s="37">
         <f t="shared" si="4"/>
-        <v>38.824000000000012</v>
+        <v>0</v>
       </c>
       <c r="AC26" s="37">
         <f t="shared" si="5"/>
-        <v>34.600000000000023</v>
+        <v>0</v>
       </c>
       <c r="AD26" s="34"/>
     </row>
@@ -3410,76 +3222,72 @@
         <v>25</v>
       </c>
       <c r="B27" s="44"/>
-      <c r="C27" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="20" t="s">
-        <v>73</v>
-      </c>
+      <c r="E27" s="20"/>
       <c r="F27" s="13">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="G27" s="22">
         <f t="shared" si="0"/>
-        <v>291.52</v>
+        <v>0</v>
       </c>
       <c r="H27" s="22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I27" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="30">
         <f t="shared" si="1"/>
-        <v>288</v>
-      </c>
-      <c r="I27" s="17">
-        <f t="shared" si="2"/>
-        <v>264</v>
-      </c>
-      <c r="J27" s="30">
-        <f t="shared" si="3"/>
-        <v>0.82499999999999996</v>
+        <v>0</v>
       </c>
       <c r="K27" s="18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L27" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M27" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="N27" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="O27" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="P27" s="18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="Q27" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="R27" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="S27" s="18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T27" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U27" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="V27" s="18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="W27" s="18">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="X27" s="18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Y27" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z27" s="18">
         <v>0</v>
@@ -3489,11 +3297,11 @@
       </c>
       <c r="AB27" s="37">
         <f t="shared" si="4"/>
-        <v>27.519999999999982</v>
+        <v>0</v>
       </c>
       <c r="AC27" s="37">
         <f t="shared" si="5"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AD27" s="34"/>
     </row>
@@ -3502,90 +3310,86 @@
         <v>26</v>
       </c>
       <c r="B28" s="44"/>
-      <c r="C28" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="20" t="s">
-        <v>74</v>
-      </c>
+      <c r="E28" s="20"/>
       <c r="F28" s="13">
-        <v>222</v>
+        <v>0</v>
       </c>
       <c r="G28" s="22">
         <f t="shared" si="0"/>
-        <v>202.24199999999999</v>
+        <v>0</v>
       </c>
       <c r="H28" s="22">
         <f>F28*90%</f>
-        <v>199.8</v>
+        <v>0</v>
       </c>
       <c r="I28" s="17">
         <f>SUM(K28:AA28)</f>
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="J28" s="30">
-        <f>I28/F28</f>
-        <v>0.97297297297297303</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="K28" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L28" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="M28" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="N28" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O28" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="P28" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q28" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="R28" s="18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="S28" s="18">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="T28" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U28" s="18">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V28" s="18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W28" s="18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="X28" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y28" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z28" s="18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA28" s="18">
         <v>0</v>
       </c>
       <c r="AB28" s="37">
         <f t="shared" si="4"/>
-        <v>-13.75800000000001</v>
+        <v>0</v>
       </c>
       <c r="AC28" s="37">
         <f t="shared" si="5"/>
-        <v>-16.199999999999989</v>
+        <v>0</v>
       </c>
       <c r="AD28" s="34"/>
     </row>
@@ -3594,79 +3398,75 @@
         <v>27</v>
       </c>
       <c r="B29" s="44"/>
-      <c r="C29" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C29" s="13"/>
       <c r="D29" s="13"/>
-      <c r="E29" s="20" t="s">
-        <v>75</v>
-      </c>
+      <c r="E29" s="20"/>
       <c r="F29" s="13">
-        <v>304</v>
+        <v>0</v>
       </c>
       <c r="G29" s="22">
         <f t="shared" si="0"/>
-        <v>276.94400000000002</v>
+        <v>0</v>
       </c>
       <c r="H29" s="22">
         <f>F29*90%</f>
-        <v>273.60000000000002</v>
+        <v>0</v>
       </c>
       <c r="I29" s="17">
         <f>SUM(K29:AA29)</f>
-        <v>245</v>
+        <v>0</v>
       </c>
       <c r="J29" s="30">
-        <f>I29/F29</f>
-        <v>0.80592105263157898</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="K29" s="18">
         <v>0</v>
       </c>
       <c r="L29" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="M29" s="18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="N29" s="18">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="O29" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="P29" s="18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q29" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="R29" s="18">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="S29" s="18">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="T29" s="18">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="U29" s="18">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="V29" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W29" s="18">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="X29" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="Y29" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z29" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA29" s="18">
         <v>0</v>
@@ -3680,90 +3480,86 @@
         <v>28</v>
       </c>
       <c r="B30" s="44"/>
-      <c r="C30" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="C30" s="13"/>
       <c r="D30" s="13"/>
-      <c r="E30" s="20" t="s">
-        <v>76</v>
-      </c>
+      <c r="E30" s="20"/>
       <c r="F30" s="13">
-        <v>274</v>
+        <v>0</v>
       </c>
       <c r="G30" s="22">
         <f t="shared" si="0"/>
-        <v>249.614</v>
+        <v>0</v>
       </c>
       <c r="H30" s="22">
         <f>F30*90%</f>
-        <v>246.6</v>
+        <v>0</v>
       </c>
       <c r="I30" s="17">
         <f>SUM(K30:AA30)</f>
-        <v>246</v>
+        <v>0</v>
       </c>
       <c r="J30" s="30">
-        <f>I30/F30</f>
-        <v>0.8978102189781022</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="K30" s="18">
         <v>0</v>
       </c>
       <c r="L30" s="18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M30" s="18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="N30" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="O30" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="P30" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q30" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="R30" s="18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="S30" s="18">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="T30" s="18">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="U30" s="18">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="V30" s="18">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="W30" s="18">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="X30" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y30" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z30" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA30" s="18">
         <v>0</v>
       </c>
       <c r="AB30" s="37">
         <f t="shared" si="4"/>
-        <v>3.6140000000000043</v>
+        <v>0</v>
       </c>
       <c r="AC30" s="37">
         <f t="shared" si="5"/>
-        <v>0.59999999999999432</v>
+        <v>0</v>
       </c>
       <c r="AD30" s="34"/>
     </row>
@@ -3777,87 +3573,87 @@
       <c r="E31" s="38"/>
       <c r="F31" s="14">
         <f>SUM(F3:F30)</f>
-        <v>6888</v>
+        <v>0</v>
       </c>
       <c r="G31" s="14">
         <f>SUM(G3:G30)</f>
-        <v>6274.9679999999998</v>
+        <v>0</v>
       </c>
       <c r="H31" s="14">
         <f>SUM(H3:H30)</f>
-        <v>6199.2000000000016</v>
+        <v>0</v>
       </c>
       <c r="I31" s="17">
         <f>SUM(K31:AA31)</f>
-        <v>6105</v>
+        <v>0</v>
       </c>
       <c r="J31" s="23">
-        <f>I31/F31</f>
-        <v>0.88632404181184665</v>
+        <f>IF(F31=0, 0, I31/F31)</f>
+        <v>0</v>
       </c>
       <c r="K31" s="19">
         <f t="shared" ref="K31:AA31" si="6">SUM(K3:K30)</f>
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="L31" s="19">
         <f t="shared" si="6"/>
-        <v>408</v>
+        <v>0</v>
       </c>
       <c r="M31" s="19">
         <f t="shared" si="6"/>
-        <v>492</v>
+        <v>0</v>
       </c>
       <c r="N31" s="19">
         <f t="shared" si="6"/>
-        <v>456</v>
+        <v>0</v>
       </c>
       <c r="O31" s="19">
         <f t="shared" si="6"/>
-        <v>520</v>
+        <v>0</v>
       </c>
       <c r="P31" s="19">
         <f t="shared" si="6"/>
-        <v>404</v>
+        <v>0</v>
       </c>
       <c r="Q31" s="19">
         <f t="shared" si="6"/>
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="R31" s="19">
         <f t="shared" si="6"/>
-        <v>486</v>
+        <v>0</v>
       </c>
       <c r="S31" s="19">
         <f t="shared" si="6"/>
-        <v>491</v>
+        <v>0</v>
       </c>
       <c r="T31" s="19">
         <f t="shared" si="6"/>
-        <v>446</v>
+        <v>0</v>
       </c>
       <c r="U31" s="19">
         <f t="shared" si="6"/>
-        <v>471</v>
+        <v>0</v>
       </c>
       <c r="V31" s="19">
         <f t="shared" si="6"/>
-        <v>415</v>
+        <v>0</v>
       </c>
       <c r="W31" s="19">
         <f t="shared" si="6"/>
-        <v>443</v>
+        <v>0</v>
       </c>
       <c r="X31" s="19">
         <f t="shared" si="6"/>
-        <v>429</v>
+        <v>0</v>
       </c>
       <c r="Y31" s="19">
         <f t="shared" si="6"/>
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="Z31" s="19">
         <f t="shared" si="6"/>
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="AA31" s="19">
         <f t="shared" si="6"/>
@@ -3865,11 +3661,11 @@
       </c>
       <c r="AB31" s="37">
         <f>G31-I31</f>
-        <v>169.96799999999985</v>
+        <v>0</v>
       </c>
       <c r="AC31" s="37">
         <f>H31-I31</f>
-        <v>94.200000000001637</v>
+        <v>0</v>
       </c>
       <c r="AD31" s="34"/>
     </row>

</xml_diff>